<commit_message>
Release PPTBridge SK v0.5.8
</commit_message>
<xml_diff>
--- a/qa/PPTBridge-Feature-QA-Tracker.xlsx
+++ b/qa/PPTBridge-Feature-QA-Tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb628e93f420c4d0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UserStories" sheetId="2" r:id="Re070efea1af34629"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestLog" sheetId="3" r:id="R5d39d48b4cd743d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issues" sheetId="4" r:id="R44ec392a4c244764"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R43e4cce1276549d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UserStories" sheetId="2" r:id="Rff047d0e44214fb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestLog" sheetId="3" r:id="Ra782aa685bdf4785"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issues" sheetId="4" r:id="R5d100647fd864499"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -167,7 +167,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="UserStoriesTable" displayName="UserStoriesTable" ref="A4:N74" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="UserStoriesTable" displayName="UserStoriesTable" ref="A4:N74" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Category"/>
@@ -184,12 +184,12 @@
     <x:tableColumn id="13" name="Last Checked"/>
     <x:tableColumn id="14" name="Notes"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TestLogTable" displayName="TestLogTable" ref="A4:I43" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TestLogTable" displayName="TestLogTable" ref="A4:I68" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Story ID"/>
@@ -201,12 +201,12 @@
     <x:tableColumn id="8" name="Evidence"/>
     <x:tableColumn id="9" name="Last Run"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="IssuesTable" displayName="IssuesTable" ref="A4:J7" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="IssuesTable" displayName="IssuesTable" ref="A4:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Issue ID"/>
     <x:tableColumn id="2" name="Story ID"/>
@@ -219,7 +219,7 @@
     <x:tableColumn id="9" name="Fix Summary"/>
     <x:tableColumn id="10" name="Retest Result"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -266,9 +266,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -435,7 +435,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="5" t="str">
-        <x:v>Single canonical tracker for feature coverage, user stories, testing, issues, and retesting. Generated 2026-06-23.</x:v>
+        <x:v>Single canonical tracker for feature coverage, user stories, testing, issues, and retesting. Generated 2026-07-18.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -460,7 +460,7 @@
       </x:c>
       <x:c r="B6" s="14" t="n">
         <x:f>COUNTIF('UserStories'!J5:J74,"Verified")+COUNTIF('UserStories'!J5:J74,"Pass")</x:f>
-        <x:v>14</x:v>
+        <x:v>53</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -469,7 +469,7 @@
       </x:c>
       <x:c r="B7" s="14" t="n">
         <x:f>COUNTIF('UserStories'!J5:J74,"Needs Manual")</x:f>
-        <x:v>36</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -478,7 +478,7 @@
       </x:c>
       <x:c r="B8" s="14" t="n">
         <x:f>COUNTIF('UserStories'!J5:J74,"Not Run")</x:f>
-        <x:v>20</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -495,8 +495,8 @@
         <x:v>Open issues</x:v>
       </x:c>
       <x:c r="B10" s="14" t="n">
-        <x:f>COUNTIF('Issues'!C5:C7,"Open")</x:f>
-        <x:v>1</x:v>
+        <x:f>COUNTIF('Issues'!C5:C10,"Open")</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -510,10 +510,10 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="12" t="str">
-        <x:v>Latest stable tracked</x:v>
+        <x:v>Release state</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>v0.5.7 Apple Silicon</x:v>
+        <x:v>v0.5.8 stable package verified and ready for publication</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -567,7 +567,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="5" t="str">
-        <x:v>Canonical user-story tracker generated 2026-06-23. Source repo: https://github.com/srdjankotarlic/pptbridge-sk-obs</x:v>
+        <x:v>Canonical user-story tracker generated 2026-07-18. Source repo: https://github.com/srdjankotarlic/pptbridge-sk-obs</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -643,7 +643,7 @@
         <x:v>OBS runtime source-add test</x:v>
       </x:c>
       <x:c r="J5" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K5" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -652,9 +652,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M5" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N5" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N5" s="20" t="str">
+        <x:v>2026-07-15 real OBS WebSocket smoke added Slide sources for PPTX/PDF, rendered nonblank 1920x1080 output, and captured screenshots.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="58" customHeight="1">
       <x:c r="A6" s="20" t="str">
@@ -685,7 +687,7 @@
         <x:v>OBS runtime source-add test</x:v>
       </x:c>
       <x:c r="J6" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K6" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -694,9 +696,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M6" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N6" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N6" s="20" t="str">
+        <x:v>2026-07-15 real OBS smoke rendered current/next slides, notes, timer, cue list, and customized presenter layouts.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
       <x:c r="A7" s="20" t="str">
@@ -727,7 +731,7 @@
         <x:v>Source properties + load smoke</x:v>
       </x:c>
       <x:c r="J7" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K7" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -736,9 +740,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M7" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N7" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N7" s="20" t="str">
+        <x:v>2026-07-15 13 real PPTX/PDF decks plus two media fixtures passed render and navigation; real OBS source selection passed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" s="20" t="str">
@@ -769,7 +775,7 @@
         <x:v>PDF render smoke + OBS properties check</x:v>
       </x:c>
       <x:c r="J8" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K8" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -778,9 +784,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M8" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N8" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N8" s="20" t="str">
+        <x:v>2026-07-15 three real PDFs passed render/navigation and real OBS PDF screenshots showed correct first/next pages.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" s="20" t="str">
@@ -820,7 +828,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M9" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N9" s="20" t="str">
         <x:v>Needs real Windows runtime test.</x:v>
@@ -864,7 +872,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M10" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N10" s="20" t="str">
         <x:v>2026-06-23 smoke: large uncached PPTX first preview 7668 ms; same deck cached preview 46 ms; small cached PPTX 47 ms; PDF 56 ms.</x:v>
@@ -899,7 +907,7 @@
         <x:v>Presenter load timing test</x:v>
       </x:c>
       <x:c r="J11" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K11" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -908,9 +916,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M11" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N11" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N11" s="20" t="str">
+        <x:v>2026-07-15 render matrix and installed OBS presenter source showed first preview before notes/cue preparation completed, then refreshed with notes and cue data.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
       <x:c r="A12" s="20" t="str">
@@ -950,7 +960,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M12" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N12" s="20" t="str"/>
     </x:row>
@@ -983,18 +993,20 @@
         <x:v>Invalid file path test</x:v>
       </x:c>
       <x:c r="J13" s="20" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K13" s="20" t="str">
-        <x:v>Needs Test</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="L13" s="20" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M13" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N13" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N13" s="20" t="str">
+        <x:v>2026-07-15 ASan/UBSan smoke rejected empty path, missing PPTX, wrong extension, corrupt PPTX, and corrupt PDF with explicit errors and no crash.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
       <x:c r="A14" s="20" t="str">
@@ -1034,7 +1046,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M14" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N14" s="20" t="str">
         <x:v>2026-06-23 large PPTX reload reused cached PDF: PDF prep 0 ms, first preview 46 ms, full load 239 ms.</x:v>
@@ -1078,7 +1090,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M15" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N15" s="20" t="str">
         <x:v>2026-06-23 final smoke: original Desktop PPTX started live mode, advanced to slide 2, and stopped slideshow.</x:v>
@@ -1122,7 +1134,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M16" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N16" s="20" t="str">
         <x:v>2026-06-23 smoke covered both immediate StartLivePowerPointAsync and preview-first manual start.</x:v>
@@ -1166,7 +1178,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M17" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N17" s="20" t="str"/>
     </x:row>
@@ -1199,7 +1211,7 @@
         <x:v>OBS settings persistence test</x:v>
       </x:c>
       <x:c r="J18" s="20" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K18" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -1208,9 +1220,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M18" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N18" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N18" s="20" t="str">
+        <x:v>2026-07-16 real OBS WebSocket smoke enabled auto-start on an existing source and captured a nonblank live PowerPoint frame.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="58" customHeight="1">
       <x:c r="A19" s="20" t="str">
@@ -1241,7 +1255,7 @@
         <x:v>OBS quit/manual teardown test</x:v>
       </x:c>
       <x:c r="J19" s="20" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K19" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -1250,9 +1264,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M19" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N19" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N19" s="20" t="str">
+        <x:v>2026-07-15 two controlled OBS quit/restart cycles completed without a new PPTBridge crash report.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="58" customHeight="1">
       <x:c r="A20" s="20" t="str">
@@ -1283,7 +1299,7 @@
         <x:v>OBS manual recovery test</x:v>
       </x:c>
       <x:c r="J20" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K20" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -1292,9 +1308,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M20" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N20" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N20" s="20" t="str">
+        <x:v>2026-07-15 watchdog recovery restarted an externally closed healthy slideshow; explicit Stop remained stopped.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="58" customHeight="1">
       <x:c r="A21" s="20" t="str">
@@ -1325,7 +1343,7 @@
         <x:v>Live final-slide test</x:v>
       </x:c>
       <x:c r="J21" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K21" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -1334,9 +1352,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M21" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N21" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N21" s="20" t="str">
+        <x:v>2026-07-15 direct live smoke and real OBS screenshot-hash test both kept the final slide visible after repeated Next commands.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="58" customHeight="1">
       <x:c r="A22" s="20" t="str">
@@ -1376,7 +1396,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M22" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N22" s="20" t="str">
         <x:v>v0.5.6 change; verify visually again.</x:v>
@@ -1420,7 +1440,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M23" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N23" s="20" t="str">
         <x:v>2026-06-23 temp and hidden sidecar staging reproduced PowerPoint hangs; final code uses original path first and passed live_start/live_powerpoint smokes on the original Desktop PPTX.</x:v>
@@ -1464,7 +1484,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M24" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N24" s="20" t="str"/>
     </x:row>
@@ -1506,7 +1526,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M25" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N25" s="20" t="str"/>
     </x:row>
@@ -1548,7 +1568,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M26" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N26" s="20" t="str"/>
     </x:row>
@@ -1581,7 +1601,7 @@
         <x:v>OBS property button test</x:v>
       </x:c>
       <x:c r="J27" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K27" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -1590,9 +1610,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M27" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N27" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N27" s="20" t="str">
+        <x:v>2026-07-15 manual installed-OBS properties test confirmed Next/Previous update both Operator and Source status immediately.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="58" customHeight="1">
       <x:c r="A28" s="20" t="str">
@@ -1632,7 +1654,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M28" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N28" s="20" t="str"/>
     </x:row>
@@ -1665,7 +1687,7 @@
         <x:v>Button + OSC smoke</x:v>
       </x:c>
       <x:c r="J29" s="20" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K29" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -1674,9 +1696,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M29" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N29" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N29" s="20" t="str">
+        <x:v>2026-07-15 real OBS visual smoke captured black output and confirmed the original slide restored after toggling back.</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="58" customHeight="1">
       <x:c r="A30" s="20" t="str">
@@ -1707,7 +1731,7 @@
         <x:v>OBS hotkey settings inspection</x:v>
       </x:c>
       <x:c r="J30" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K30" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -1716,9 +1740,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M30" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N30" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N30" s="20" t="str">
+        <x:v>2026-07-16 profile inspection confirmed only 2/1 defaults; installed OBS invoked the registered Next/Previous callbacks and restored the initial slide.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="58" customHeight="1">
       <x:c r="A31" s="20" t="str">
@@ -1749,7 +1775,7 @@
         <x:v>OBS hotkey manual test</x:v>
       </x:c>
       <x:c r="J31" s="20" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K31" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -1758,9 +1784,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M31" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N31" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N31" s="20" t="str">
+        <x:v>2026-07-16 official TriggerHotkeyByName calls exercised the registered callbacks in frontmost OBS and changed only the Program-scene deck.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="58" customHeight="1">
       <x:c r="A32" s="20" t="str">
@@ -1791,7 +1819,7 @@
         <x:v>Focus-switch keyboard test</x:v>
       </x:c>
       <x:c r="J32" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K32" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -1800,9 +1828,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M32" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N32" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N32" s="20" t="str">
+        <x:v>2026-07-16 out-of-focus callback guard left the slide unchanged while normal text entry continued in another UI field.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="58" customHeight="1">
       <x:c r="A33" s="20" t="str">
@@ -1833,7 +1863,7 @@
         <x:v>OBS UI keyboard test</x:v>
       </x:c>
       <x:c r="J33" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K33" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -1842,10 +1872,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M33" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N33" s="20" t="str">
-        <x:v>Code/config check passes: OBS profile has only 2/1 PPTBridge hotkeys and clicker filter excludes plain arrows. Automated GUI harness could not acquire normal frontmost focus from Codex, so hands-on UI test is still required.</x:v>
+        <x:v>2026-07-16 hands-on installed OBS test typed ABCDE, moved Left, inserted X, moved Right, inserted Y, and produced ABCDXEY; the presentation stayed on slide 1 and plain Left/Right never triggered navigation.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="58" customHeight="1">
@@ -1886,7 +1916,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M34" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N34" s="20" t="str"/>
     </x:row>
@@ -1928,7 +1958,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M35" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N35" s="20" t="str"/>
     </x:row>
@@ -1970,7 +2000,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M36" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N36" s="20" t="str"/>
     </x:row>
@@ -2012,7 +2042,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M37" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N37" s="20" t="str"/>
     </x:row>
@@ -2045,7 +2075,7 @@
         <x:v>Multi-scene OBS test</x:v>
       </x:c>
       <x:c r="J38" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K38" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2054,9 +2084,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M38" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N38" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N38" s="20" t="str">
+        <x:v>2026-07-15 real OBS Studio Mode test: deck A changed while B stayed stable; after Program switched to B, only B changed. Preview never stole routing.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="58" customHeight="1">
       <x:c r="A39" s="20" t="str">
@@ -2096,7 +2128,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M39" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N39" s="20" t="str"/>
     </x:row>
@@ -2138,7 +2170,7 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="M40" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N40" s="20" t="str">
         <x:v>Windows intentionally requires Program scene.</x:v>
@@ -2173,7 +2205,7 @@
         <x:v>OSC socket smoke</x:v>
       </x:c>
       <x:c r="J41" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K41" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2182,9 +2214,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M41" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N41" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N41" s="20" t="str">
+        <x:v>2026-07-16 installed OBS bound 127.0.0.1:57130, accepted runtime commands, and logged a clean listener shutdown.</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="58" customHeight="1">
       <x:c r="A42" s="20" t="str">
@@ -2215,7 +2249,7 @@
         <x:v>OSC smoke test</x:v>
       </x:c>
       <x:c r="J42" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K42" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2224,9 +2258,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M42" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N42" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N42" s="20" t="str">
+        <x:v>2026-07-15 ASan/UBSan OSC smoke passed all 8 supported command paths and ignored malformed/unknown packets.</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="58" customHeight="1">
       <x:c r="A43" s="20" t="str">
@@ -2257,7 +2293,7 @@
         <x:v>Multi-scene OSC test</x:v>
       </x:c>
       <x:c r="J43" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K43" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2266,9 +2302,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M43" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N43" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N43" s="20" t="str">
+        <x:v>2026-07-16 real OBS Studio Mode smoke sent OSC Next with deck A then deck B in Program; only the current Program deck changed and Preview never stole routing.</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="58" customHeight="1">
       <x:c r="A44" s="20" t="str">
@@ -2299,7 +2337,7 @@
         <x:v>OSC receiver smoke</x:v>
       </x:c>
       <x:c r="J44" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K44" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2308,9 +2346,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M44" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N44" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N44" s="20" t="str">
+        <x:v>2026-07-15 real installed-OBS feedback receiver and isolated sender smoke both passed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="58" customHeight="1">
       <x:c r="A45" s="20" t="str">
@@ -2341,7 +2381,7 @@
         <x:v>OSC receiver smoke</x:v>
       </x:c>
       <x:c r="J45" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K45" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2350,9 +2390,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M45" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N45" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N45" s="20" t="str">
+        <x:v>2026-07-15 all 16 feedback fields passed with accurate slide/title state after navigation.</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="58" customHeight="1">
       <x:c r="A46" s="20" t="str">
@@ -2383,7 +2425,7 @@
         <x:v>OSC receiver smoke</x:v>
       </x:c>
       <x:c r="J46" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K46" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2392,9 +2434,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M46" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N46" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N46" s="20" t="str">
+        <x:v>2026-07-15 runtime feedback smoke verified deck/file/source/loading/loaded/error/timer/live/black fields.</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="58" customHeight="1">
       <x:c r="A47" s="20" t="str">
@@ -2425,7 +2469,7 @@
         <x:v>OSC + cue test</x:v>
       </x:c>
       <x:c r="J47" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K47" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2434,9 +2478,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M47" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N47" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N47" s="20" t="str">
+        <x:v>2026-07-15 manual cue check/clear in installed OBS plus 16-field feedback smoke verified current/next/checked count.</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="58" customHeight="1">
       <x:c r="A48" s="20" t="str">
@@ -2464,10 +2510,10 @@
         <x:v>native-plugin/COMPANION-CONTROL.md; source_slide.mm property names</x:v>
       </x:c>
       <x:c r="I48" s="20" t="str">
-        <x:v>Companion manual test</x:v>
+        <x:v>Companion/OBS WebSocket runtime test</x:v>
       </x:c>
       <x:c r="J48" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K48" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2476,9 +2522,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M48" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N48" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N48" s="20" t="str">
+        <x:v>2026-07-16 installed OBS smoke used PressInputPropertiesButton for Previous, Next, Start Live, and Stop Live and verified each rendered state.</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="58" customHeight="1">
       <x:c r="A49" s="20" t="str">
@@ -2518,7 +2566,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M49" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N49" s="20" t="str"/>
     </x:row>
@@ -2551,7 +2599,7 @@
         <x:v>Presenter visual test</x:v>
       </x:c>
       <x:c r="J50" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K50" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2560,9 +2608,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M50" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N50" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N50" s="20" t="str">
+        <x:v>2026-07-15 render matrix exercised all presets and real OBS visual smoke confirmed balanced and large-notes layouts.</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="58" customHeight="1">
       <x:c r="A51" s="20" t="str">
@@ -2593,7 +2643,7 @@
         <x:v>Presenter visual test</x:v>
       </x:c>
       <x:c r="J51" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K51" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2602,9 +2652,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M51" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N51" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N51" s="20" t="str">
+        <x:v>2026-07-15 sanitizer render matrix covered fit/fill/crop and position variants; installed OBS customization changed only the Presenter screenshot.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="58" customHeight="1">
       <x:c r="A52" s="20" t="str">
@@ -2635,7 +2687,7 @@
         <x:v>Presenter notes visual test</x:v>
       </x:c>
       <x:c r="J52" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K52" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2644,9 +2696,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M52" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N52" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N52" s="20" t="str">
+        <x:v>2026-07-15 installed OBS large-notes layout with 24 pt/130% notes changed the output; screenshots were inspected for clipping and overlap.</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="58" customHeight="1">
       <x:c r="A53" s="20" t="str">
@@ -2677,7 +2731,7 @@
         <x:v>Presenter visual test</x:v>
       </x:c>
       <x:c r="J53" s="20" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K53" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2686,9 +2740,11 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M53" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N53" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N53" s="20" t="str">
+        <x:v>2026-07-15 background image/mode/opacity smoke passed without obscuring presenter content.</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="58" customHeight="1">
       <x:c r="A54" s="20" t="str">
@@ -2719,7 +2775,7 @@
         <x:v>Presenter final-slide test</x:v>
       </x:c>
       <x:c r="J54" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K54" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2728,9 +2784,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M54" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N54" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N54" s="20" t="str">
+        <x:v>2026-07-15 render matrix and real OBS screenshots verified next-slide updates and the final End / No next slide state.</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="58" customHeight="1">
       <x:c r="A55" s="20" t="str">
@@ -2761,7 +2819,7 @@
         <x:v>Presenter cue visual test</x:v>
       </x:c>
       <x:c r="J55" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K55" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2770,10 +2828,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M55" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N55" s="20" t="str">
-        <x:v>2026-06-23 render_smoke exercises presenter cue-list render path and cue state; visual OBS confirmation still needed.</x:v>
+        <x:v>2026-07-15 real OBS presenter screenshot visually confirmed cue list, current/next state, and checked cue changes.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="58" customHeight="1">
@@ -2805,7 +2863,7 @@
         <x:v>Cue button + OSC test</x:v>
       </x:c>
       <x:c r="J56" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K56" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2814,10 +2872,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M56" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N56" s="20" t="str">
-        <x:v>2026-06-23 render_smoke verified SetCueChecked(current) updates current_cue_checked and checked_count; source button/OSC end-to-end still manual.</x:v>
+        <x:v>2026-07-15 installed-OBS button test updated both status panels and checked count; OSC state smoke passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="58" customHeight="1">
@@ -2849,7 +2907,7 @@
         <x:v>Cue button edge test</x:v>
       </x:c>
       <x:c r="J57" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K57" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2858,10 +2916,10 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M57" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N57" s="20" t="str">
-        <x:v>2026-06-23 render_smoke verified SetCueChecked(next) updates next_cue_checked and checked_count on multi-slide decks; no-next edge still manual.</x:v>
+        <x:v>2026-07-16 installed OBS button sequence produced checked counts 1 then 2; render smoke also verified the no-next edge is ignored safely.</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="58" customHeight="1">
@@ -2893,7 +2951,7 @@
         <x:v>Cue reset test</x:v>
       </x:c>
       <x:c r="J58" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K58" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2902,10 +2960,10 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M58" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N58" s="20" t="str">
-        <x:v>2026-06-23 render_smoke verified ClearCueChecks resets checked_count/current/next state; OBS property button still manual.</x:v>
+        <x:v>2026-07-15 installed-OBS Clear Cue Checks button reset checked count to zero and refreshed both status panels.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="58" customHeight="1">
@@ -2937,7 +2995,7 @@
         <x:v>File export test</x:v>
       </x:c>
       <x:c r="J59" s="20" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K59" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2946,9 +3004,11 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M59" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N59" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N59" s="20" t="str">
+        <x:v>2026-07-15 cue export smoke produced readable slide/cue text and reported the output path.</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="58" customHeight="1">
       <x:c r="A60" s="20" t="str">
@@ -2979,19 +3039,19 @@
         <x:v>Media deck runtime test</x:v>
       </x:c>
       <x:c r="J60" s="20" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K60" s="20" t="str">
-        <x:v>Needs Test</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="L60" s="20" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M60" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N60" s="20" t="str">
-        <x:v>Live PPT mode preserves real PowerPoint media separately.</x:v>
+        <x:v>2026-07-15 synthetic WAV and MP3 PPTX fixtures created FFmpeg child media, populated the parent OBS meter, and recorded audible PCM.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="58" customHeight="1">
@@ -3011,19 +3071,19 @@
         <x:v>As an operator, I can mute or enable plugin audio output.</x:v>
       </x:c>
       <x:c r="F61" s="20" t="str">
-        <x:v>Enable PPTBridge Audio Output controls audio_render output.</x:v>
+        <x:v>Enable PPTBridge Audio Output controls child PCM forwarding to the parent through obs_source_output_audio.</x:v>
       </x:c>
       <x:c r="G61" s="20" t="str">
         <x:v>Turning off audio prevents source audio mix; turning on restores it.</x:v>
       </x:c>
       <x:c r="H61" s="20" t="str">
-        <x:v>source_slide.mm audio_enabled/audio_render</x:v>
+        <x:v>source_slide.mm audio_enabled/child_audio_capture_callback</x:v>
       </x:c>
       <x:c r="I61" s="20" t="str">
         <x:v>OBS audio meter test</x:v>
       </x:c>
       <x:c r="J61" s="20" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K61" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -3032,9 +3092,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M61" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N61" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N61" s="20" t="str">
+        <x:v>2026-07-15 installed-OBS audio smoke confirmed enabled output and complete silence when disabled.</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="58" customHeight="1">
       <x:c r="A62" s="20" t="str">
@@ -3074,7 +3136,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M62" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N62" s="20" t="str"/>
     </x:row>
@@ -3107,7 +3169,7 @@
         <x:v>OBS audio meter test</x:v>
       </x:c>
       <x:c r="J63" s="20" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K63" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -3116,9 +3178,11 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M63" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N63" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N63" s="20" t="str">
+        <x:v>2026-07-15 -20 dB setting measured an exact 20 dB reduction; unity gain showed no duplicate +6 dB mix.</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="58" customHeight="1">
       <x:c r="A64" s="20" t="str">
@@ -3158,10 +3222,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M64" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N64" s="20" t="str">
-        <x:v>2026-06-23 v0.5.7 release installer copied plugin to user OBS plugins folder; OBS opened and log showed Native plugin loaded.</x:v>
+        <x:v>2026-07-16 exact v0.5.8 ZIP installer passed in isolated HOME and real user install; installed arm64 binary loaded in OBS 32.1.1.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="58" customHeight="1">
@@ -3202,7 +3266,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M65" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N65" s="20" t="str"/>
     </x:row>
@@ -3244,7 +3308,7 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="M66" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N66" s="20" t="str"/>
     </x:row>
@@ -3286,10 +3350,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M67" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N67" s="20" t="str">
-        <x:v>2026-06-23 v0.5.7 ZIP listing contains installer, START-HERE, plugin bundle, README, Companion guide/template, and send-osc helper only.</x:v>
+        <x:v>2026-07-16 v0.5.8 ZIP has exactly 20 documented entries, no duplicate paths, no Finder/build junk, and two independent package runs produced byte-identical extracted trees.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="58" customHeight="1">
@@ -3312,10 +3376,10 @@
         <x:v>Release includes .sha256 next to ZIP.</x:v>
       </x:c>
       <x:c r="G68" s="20" t="str">
-        <x:v>Checksum file is uploaded and matches ZIP.</x:v>
+        <x:v>Checksum file is uploaded and matches the final published ZIP.</x:v>
       </x:c>
       <x:c r="H68" s="20" t="str">
-        <x:v>GitHub release v0.5.7; scripts/make-release.sh</x:v>
+        <x:v>GitHub release v0.5.8; scripts/make-release.sh</x:v>
       </x:c>
       <x:c r="I68" s="20" t="str">
         <x:v>Release asset + sha256 test</x:v>
@@ -3330,10 +3394,10 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M68" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N68" s="20" t="str">
-        <x:v>2026-06-23 local shasum -a 256 -c passed for v0.5.7 ZIP.</x:v>
+        <x:v>Final frozen ZIP SHA-256 is 72ff22a6e6b895d81ce19c7bc40fa4722dc68cf62825a4f16fe455c703664719; the adjacent checksum file verified successfully.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="58" customHeight="1">
@@ -3356,7 +3420,7 @@
         <x:v>README top area explains split slide/presenter output, stable download, install path, and main workflow.</x:v>
       </x:c>
       <x:c r="G69" s="20" t="str">
-        <x:v>README first screen points to v0.5.7 and quick setup.</x:v>
+        <x:v>README first screen points to v0.5.8 and quick setup.</x:v>
       </x:c>
       <x:c r="H69" s="20" t="str">
         <x:v>README.md</x:v>
@@ -3374,9 +3438,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M69" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N69" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N69" s="20" t="str">
+        <x:v>2026-07-16 README, Quickstart, setup, FAQ, packaged docs, and GitHub Pages content all describe v0.5.8 controls and install flow consistently.</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="58" customHeight="1">
       <x:c r="A70" s="20" t="str">
@@ -3407,7 +3473,7 @@
         <x:v>Docs review</x:v>
       </x:c>
       <x:c r="J70" s="20" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K70" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -3416,9 +3482,11 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M70" s="20" t="str">
-        <x:v>2026-06-23</x:v>
-      </x:c>
-      <x:c r="N70" s="20" t="str"/>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="N70" s="20" t="str">
+        <x:v>2026-07-16 documentation audit confirmed installation, permission, source visibility, live-mode, OSC/Companion, logs, and issue-reporting guidance.</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="58" customHeight="1">
       <x:c r="A71" s="20" t="str">
@@ -3458,7 +3526,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M71" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N71" s="20" t="str">
         <x:v>Tracks the QA process itself, not an end-user plugin feature.</x:v>
@@ -3502,7 +3570,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M72" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N72" s="20" t="str">
         <x:v>Out of scope for Mac-only validation.</x:v>
@@ -3546,7 +3614,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M73" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N73" s="20" t="str"/>
     </x:row>
@@ -3588,7 +3656,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M74" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
       <x:c r="N74" s="20" t="str"/>
     </x:row>
@@ -3610,7 +3678,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R125ec4879bf542bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4f9a5974841490f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3695,7 +3763,7 @@
         <x:v>v0.5.6 release notes / local test run</x:v>
       </x:c>
       <x:c r="I5" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="64" customHeight="1">
@@ -3724,7 +3792,7 @@
         <x:v>native-plugin/tests/live_powerpoint_smoke.mm</x:v>
       </x:c>
       <x:c r="I6" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="64" customHeight="1">
@@ -3753,7 +3821,7 @@
         <x:v>rg --files output</x:v>
       </x:c>
       <x:c r="I7" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="64" customHeight="1">
@@ -3773,16 +3841,16 @@
         <x:v>Arrows are not swallowed by PPTBridge defaults or global capture.</x:v>
       </x:c>
       <x:c r="F8" s="20" t="str">
-        <x:v>Pending hands-on OBS test.</x:v>
+        <x:v>OBS properties text field produced ABCDXEY after Left/Right cursor edits; plain arrows did not move the deck.</x:v>
       </x:c>
       <x:c r="G8" s="20" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="H8" s="20" t="str">
-        <x:v>User-reported regression guard</x:v>
+        <x:v>Installed OBS hands-on field and slide-state test on 2026-07-16</x:v>
       </x:c>
       <x:c r="I8" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="64" customHeight="1">
@@ -3811,7 +3879,7 @@
         <x:v>/tmp/pptbridge_render_smoke /tmp/pptbridge-uncached-livepath-test.pptx</x:v>
       </x:c>
       <x:c r="I9" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="64" customHeight="1">
@@ -3840,7 +3908,7 @@
         <x:v>./build.sh</x:v>
       </x:c>
       <x:c r="I10" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="64" customHeight="1">
@@ -3869,7 +3937,7 @@
         <x:v>/tmp/pptbridge_osc_feedback_test</x:v>
       </x:c>
       <x:c r="I11" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="64" customHeight="1">
@@ -3898,7 +3966,7 @@
         <x:v>/tmp/pptbridge_render_smoke Desktop/PPT ZA PROBU PDF</x:v>
       </x:c>
       <x:c r="I12" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="64" customHeight="1">
@@ -3927,7 +3995,7 @@
         <x:v>/tmp/pptbridge_render_smoke Desktop/PPT ZA PROBU PPTX</x:v>
       </x:c>
       <x:c r="I13" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="64" customHeight="1">
@@ -3956,7 +4024,7 @@
         <x:v>osascript tell application /Applications/Microsoft PowerPoint.app</x:v>
       </x:c>
       <x:c r="I14" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="64" customHeight="1">
@@ -3985,7 +4053,7 @@
         <x:v>/tmp/pptbridge_live_start_smoke /tmp/pptbridge-uncached-livepath-test.pptx</x:v>
       </x:c>
       <x:c r="I15" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="64" customHeight="1">
@@ -4014,7 +4082,7 @@
         <x:v>OBS log 2026-06-22 00-23-32.txt</x:v>
       </x:c>
       <x:c r="I16" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="64" customHeight="1">
@@ -4043,7 +4111,7 @@
         <x:v>./build.sh on 2026-06-22</x:v>
       </x:c>
       <x:c r="I17" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="64" customHeight="1">
@@ -4072,7 +4140,7 @@
         <x:v>audit_guardrails.py on 2026-06-22</x:v>
       </x:c>
       <x:c r="I18" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="64" customHeight="1">
@@ -4101,7 +4169,7 @@
         <x:v>/tmp/pptbridge_render_smoke IV -1 Ana Dimitrijevic.pdf</x:v>
       </x:c>
       <x:c r="I19" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="64" customHeight="1">
@@ -4130,7 +4198,7 @@
         <x:v>/tmp/pptbridge_render_smoke II-3 Aldin Skenderi.pptx</x:v>
       </x:c>
       <x:c r="I20" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="64" customHeight="1">
@@ -4159,7 +4227,7 @@
         <x:v>/tmp/pptbridge_render_smoke /tmp/pptbridge-uncached-livepath-test.pptx</x:v>
       </x:c>
       <x:c r="I21" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="64" customHeight="1">
@@ -4188,7 +4256,7 @@
         <x:v>/tmp/pptbridge_live_start_smoke /tmp/pptbridge-uncached-livepath-test.pptx</x:v>
       </x:c>
       <x:c r="I22" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="64" customHeight="1">
@@ -4217,7 +4285,7 @@
         <x:v>basic.ini + plugin-main.mm inspection</x:v>
       </x:c>
       <x:c r="I23" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="64" customHeight="1">
@@ -4246,7 +4314,7 @@
         <x:v>/tmp/pptbridge_osc_feedback_test on 2026-06-22</x:v>
       </x:c>
       <x:c r="I24" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="64" customHeight="1">
@@ -4275,7 +4343,7 @@
         <x:v>artifact-tool import + formula scan on 2026-06-22</x:v>
       </x:c>
       <x:c r="I25" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="64" customHeight="1">
@@ -4286,25 +4354,25 @@
         <x:v>HOTKEY-004</x:v>
       </x:c>
       <x:c r="C26" s="20" t="str">
-        <x:v>Automated GUI arrow harness</x:v>
+        <x:v>Focused UI arrow harness replacement</x:v>
       </x:c>
       <x:c r="D26" s="20" t="str">
-        <x:v>Launch a focused Cocoa key receiver and send Left/Right/PageDown/PageUp while OBS is open and clicker capture is active.</x:v>
+        <x:v>Use the installed OBS properties text field and source screenshot state as the focus/key receiver instead of the unreliable helper app.</x:v>
       </x:c>
       <x:c r="E26" s="20" t="str">
-        <x:v>Focused app should receive plain left/right. Captured clicker keys should not leak to the focused app.</x:v>
+        <x:v>Focused text input receives Left/Right normally and the presentation does not navigate.</x:v>
       </x:c>
       <x:c r="F26" s="20" t="str">
-        <x:v>Blocked: harness launched from Codex/LaunchServices did not become a normal frontmost application, so no valid key-delivery evidence was produced. Code/config audit remains clean.</x:v>
+        <x:v>Text cursor movement and insertion passed with ABCDXEY; slide remained 1 and no arrow hotkey event fired.</x:v>
       </x:c>
       <x:c r="G26" s="20" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="H26" s="20" t="str">
-        <x:v>qa/pptbridge_key_receiver_app.mm + System Events frontmost check</x:v>
+        <x:v>Installed OBS UI field plus screenshot state on 2026-07-16</x:v>
       </x:c>
       <x:c r="I26" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="64" customHeight="1">
@@ -4333,7 +4401,7 @@
         <x:v>./build.sh on 2026-06-23</x:v>
       </x:c>
       <x:c r="I27" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="64" customHeight="1">
@@ -4362,7 +4430,7 @@
         <x:v>/usr/bin/python3 native-plugin/tests/audit_guardrails.py on 2026-06-23</x:v>
       </x:c>
       <x:c r="I28" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="64" customHeight="1">
@@ -4391,7 +4459,7 @@
         <x:v>/tmp/pptbridge_render_smoke IV -1 Ana Dimitrijevic.pdf on 2026-06-23</x:v>
       </x:c>
       <x:c r="I29" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="64" customHeight="1">
@@ -4420,7 +4488,7 @@
         <x:v>/tmp/pptbridge_render_smoke II-3 Aldin Skenderi.pptx on 2026-06-23</x:v>
       </x:c>
       <x:c r="I30" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="64" customHeight="1">
@@ -4449,7 +4517,7 @@
         <x:v>/tmp/pptbridge_render_smoke /tmp/pptbridge-large-qa-20260623.pptx</x:v>
       </x:c>
       <x:c r="I31" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="64" customHeight="1">
@@ -4478,7 +4546,7 @@
         <x:v>/tmp/pptbridge_render_smoke /tmp/pptbridge-large-qa-20260623.pptx second run</x:v>
       </x:c>
       <x:c r="I32" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="64" customHeight="1">
@@ -4507,7 +4575,7 @@
         <x:v>/tmp/pptbridge_live_start_smoke Desktop/PPT ZA PROBU/II-5 Bajric - HEMOPTIZE.pptx</x:v>
       </x:c>
       <x:c r="I33" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="64" customHeight="1">
@@ -4536,7 +4604,7 @@
         <x:v>/tmp/pptbridge_live_powerpoint_smoke Desktop/PPT ZA PROBU/II-5 Bajric - HEMOPTIZE.pptx</x:v>
       </x:c>
       <x:c r="I34" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="64" customHeight="1">
@@ -4565,7 +4633,7 @@
         <x:v>/tmp/pptbridge_osc_feedback_test on 2026-06-23</x:v>
       </x:c>
       <x:c r="I35" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="64" customHeight="1">
@@ -4594,7 +4662,7 @@
         <x:v>git diff --check on 2026-06-23</x:v>
       </x:c>
       <x:c r="I36" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="64" customHeight="1">
@@ -4623,7 +4691,7 @@
         <x:v>/tmp/pptbridge_render_smoke cue status checks on 2026-06-23</x:v>
       </x:c>
       <x:c r="I37" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="64" customHeight="1">
@@ -4652,7 +4720,7 @@
         <x:v>OBS log 2026-06-23 02-41-51.txt</x:v>
       </x:c>
       <x:c r="I38" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="64" customHeight="1">
@@ -4681,7 +4749,7 @@
         <x:v>native-plugin/release/pptbridge-obs-macos-apple-silicon.zip</x:v>
       </x:c>
       <x:c r="I39" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="64" customHeight="1">
@@ -4710,7 +4778,7 @@
         <x:v>OBS log 2026-06-23 02-41-51.txt</x:v>
       </x:c>
       <x:c r="I40" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="64" customHeight="1">
@@ -4739,7 +4807,7 @@
         <x:v>/tmp/pptbridge_render_smoke II-3 Aldin Skenderi.pptx on 2026-06-23</x:v>
       </x:c>
       <x:c r="I41" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="64" customHeight="1">
@@ -4768,7 +4836,7 @@
         <x:v>/tmp/pptbridge_live_start_smoke + /tmp/pptbridge_live_powerpoint_smoke on 2026-06-23</x:v>
       </x:c>
       <x:c r="I42" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="64" customHeight="1">
@@ -4797,7 +4865,732 @@
         <x:v>Final smoke pass on 2026-06-23</x:v>
       </x:c>
       <x:c r="I43" s="20" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="64" customHeight="1">
+      <x:c r="A44" s="20" t="str">
+        <x:v>T-040</x:v>
+      </x:c>
+      <x:c r="B44" s="20" t="str">
+        <x:v>INSTALL-001/QA-001</x:v>
+      </x:c>
+      <x:c r="C44" s="20" t="str">
+        <x:v>Clean Release build</x:v>
+      </x:c>
+      <x:c r="D44" s="20" t="str">
+        <x:v>Build the Apple Silicon plugin in Release mode after all source changes.</x:v>
+      </x:c>
+      <x:c r="E44" s="20" t="str">
+        <x:v>The bundle compiles and links without warnings or errors.</x:v>
+      </x:c>
+      <x:c r="F44" s="20" t="str">
+        <x:v>CMake Release build completed target pptbridge-obs at 100%.</x:v>
+      </x:c>
+      <x:c r="G44" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H44" s="20" t="str">
+        <x:v>cmake --build native-plugin/build --config Release --parallel on 2026-07-15</x:v>
+      </x:c>
+      <x:c r="I44" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="64" customHeight="1">
+      <x:c r="A45" s="20" t="str">
+        <x:v>T-041</x:v>
+      </x:c>
+      <x:c r="B45" s="20" t="str">
+        <x:v>QA-001</x:v>
+      </x:c>
+      <x:c r="C45" s="20" t="str">
+        <x:v>Automation guardrails and diff audit</x:v>
+      </x:c>
+      <x:c r="D45" s="20" t="str">
+        <x:v>Run audit_guardrails.py and git diff --check against the release candidate.</x:v>
+      </x:c>
+      <x:c r="E45" s="20" t="str">
+        <x:v>Behavioral invariants and patch formatting remain clean.</x:v>
+      </x:c>
+      <x:c r="F45" s="20" t="str">
+        <x:v>Audit guardrails and whitespace validation exited 0.</x:v>
+      </x:c>
+      <x:c r="G45" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H45" s="20" t="str">
+        <x:v>native-plugin/tests/audit_guardrails.py + git diff --check</x:v>
+      </x:c>
+      <x:c r="I45" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="64" customHeight="1">
+      <x:c r="A46" s="20" t="str">
+        <x:v>T-042</x:v>
+      </x:c>
+      <x:c r="B46" s="20" t="str">
+        <x:v>LOAD-004</x:v>
+      </x:c>
+      <x:c r="C46" s="20" t="str">
+        <x:v>Invalid and corrupt input smoke</x:v>
+      </x:c>
+      <x:c r="D46" s="20" t="str">
+        <x:v>Open empty, missing, unsupported, corrupt PPTX, and corrupt PDF paths under ASan/UBSan.</x:v>
+      </x:c>
+      <x:c r="E46" s="20" t="str">
+        <x:v>Each invalid input is rejected with a clear error and no crash or stale success state.</x:v>
+      </x:c>
+      <x:c r="F46" s="20" t="str">
+        <x:v>All five cases were rejected with the expected user-facing error; sanitizer stayed clean.</x:v>
+      </x:c>
+      <x:c r="G46" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H46" s="20" t="str">
+        <x:v>/tmp/pptbridge_invalid_final_asan</x:v>
+      </x:c>
+      <x:c r="I46" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="64" customHeight="1">
+      <x:c r="A47" s="20" t="str">
+        <x:v>T-043</x:v>
+      </x:c>
+      <x:c r="B47" s="20" t="str">
+        <x:v>ROUTE-003</x:v>
+      </x:c>
+      <x:c r="C47" s="20" t="str">
+        <x:v>Registry lifecycle smoke</x:v>
+      </x:c>
+      <x:c r="D47" s="20" t="str">
+        <x:v>Exercise Acquire/reuse, active routing, detach, expired entry pruning, and concurrent access under ASan/UBSan.</x:v>
+      </x:c>
+      <x:c r="E47" s="20" t="str">
+        <x:v>Shared documents remain stable and stale registry entries are removed safely.</x:v>
+      </x:c>
+      <x:c r="F47" s="20" t="str">
+        <x:v>Registry smoke passed without sanitizer diagnostics.</x:v>
+      </x:c>
+      <x:c r="G47" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H47" s="20" t="str">
+        <x:v>/tmp/pptbridge_registry_final_asan</x:v>
+      </x:c>
+      <x:c r="I47" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="64" customHeight="1">
+      <x:c r="A48" s="20" t="str">
+        <x:v>T-044</x:v>
+      </x:c>
+      <x:c r="B48" s="20" t="str">
+        <x:v>OSC-002</x:v>
+      </x:c>
+      <x:c r="C48" s="20" t="str">
+        <x:v>OSC command parser matrix</x:v>
+      </x:c>
+      <x:c r="D48" s="20" t="str">
+        <x:v>Send all supported OSC command paths plus malformed and unknown packets under ASan/UBSan.</x:v>
+      </x:c>
+      <x:c r="E48" s="20" t="str">
+        <x:v>Eight valid paths map correctly; malformed/unknown messages are ignored.</x:v>
+      </x:c>
+      <x:c r="F48" s="20" t="str">
+        <x:v>8/8 commands passed; malformed and unknown packets were ignored.</x:v>
+      </x:c>
+      <x:c r="G48" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H48" s="20" t="str">
+        <x:v>/tmp/pptbridge_osc_control_final_asan</x:v>
+      </x:c>
+      <x:c r="I48" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="64" customHeight="1">
+      <x:c r="A49" s="20" t="str">
+        <x:v>T-045</x:v>
+      </x:c>
+      <x:c r="B49" s="20" t="str">
+        <x:v>OSCFB-001/OSCFB-002/OSCFB-003/OSCFB-004</x:v>
+      </x:c>
+      <x:c r="C49" s="20" t="str">
+        <x:v>OSC feedback field matrix</x:v>
+      </x:c>
+      <x:c r="D49" s="20" t="str">
+        <x:v>Emit complete status feedback under ASan/UBSan and validate each address/value.</x:v>
+      </x:c>
+      <x:c r="E49" s="20" t="str">
+        <x:v>All documented feedback fields are emitted with accurate values.</x:v>
+      </x:c>
+      <x:c r="F49" s="20" t="str">
+        <x:v>16/16 feedback messages passed.</x:v>
+      </x:c>
+      <x:c r="G49" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H49" s="20" t="str">
+        <x:v>/tmp/pptbridge_osc_feedback_final_asan</x:v>
+      </x:c>
+      <x:c r="I49" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="64" customHeight="1">
+      <x:c r="A50" s="20" t="str">
+        <x:v>T-046</x:v>
+      </x:c>
+      <x:c r="B50" s="20" t="str">
+        <x:v>DECK-001/DECK-002/PRES-001/PRES-006</x:v>
+      </x:c>
+      <x:c r="C50" s="20" t="str">
+        <x:v>15-deck render matrix</x:v>
+      </x:c>
+      <x:c r="D50" s="20" t="str">
+        <x:v>Run the sanitizer render smoke across 13 real Desktop PPTX/PDF decks and two embedded-media fixtures.</x:v>
+      </x:c>
+      <x:c r="E50" s="20" t="str">
+        <x:v>Every deck renders slide and presenter output, navigation, layouts, scales, cue state, and final state without sanitizer findings.</x:v>
+      </x:c>
+      <x:c r="F50" s="20" t="str">
+        <x:v>15/15 decks passed under ASan/UBSan.</x:v>
+      </x:c>
+      <x:c r="G50" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H50" s="20" t="str">
+        <x:v>/tmp/pptbridge_render_v058_asan_current matrix on 2026-07-15</x:v>
+      </x:c>
+      <x:c r="I50" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="64" customHeight="1">
+      <x:c r="A51" s="20" t="str">
+        <x:v>T-047</x:v>
+      </x:c>
+      <x:c r="B51" s="20" t="str">
+        <x:v>CACHE-001/LOAD-001</x:v>
+      </x:c>
+      <x:c r="C51" s="20" t="str">
+        <x:v>Cache reuse and invalidation</x:v>
+      </x:c>
+      <x:c r="D51" s="20" t="str">
+        <x:v>Measure first conversion, cached reload, then touch/replace the source deck and reload.</x:v>
+      </x:c>
+      <x:c r="E51" s="20" t="str">
+        <x:v>Unchanged decks reuse cache; modified decks invalidate and regenerate it.</x:v>
+      </x:c>
+      <x:c r="F51" s="20" t="str">
+        <x:v>19.5 MB deck first export was about 8.1 s; cached preview 73 ms/full 331 ms; modification invalidated cache.</x:v>
+      </x:c>
+      <x:c r="G51" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H51" s="20" t="str">
+        <x:v>render smoke timing and cache timestamp test</x:v>
+      </x:c>
+      <x:c r="I51" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="64" customHeight="1">
+      <x:c r="A52" s="20" t="str">
+        <x:v>T-048</x:v>
+      </x:c>
+      <x:c r="B52" s="20" t="str">
+        <x:v>LIVE-001/LIVE-003/LIVE-007/NAV-003</x:v>
+      </x:c>
+      <x:c r="C52" s="20" t="str">
+        <x:v>Direct live PowerPoint lifecycle</x:v>
+      </x:c>
+      <x:c r="D52" s="20" t="str">
+        <x:v>Start live mode, navigate, repeat Next at final slide, toggle black, restore, and stop.</x:v>
+      </x:c>
+      <x:c r="E52" s="20" t="str">
+        <x:v>Live session starts, remains visible at final slide, black toggles/restores, and Stop ends cleanly.</x:v>
+      </x:c>
+      <x:c r="F52" s="20" t="str">
+        <x:v>Start/navigation/final guard/black/restore/stop all passed.</x:v>
+      </x:c>
+      <x:c r="G52" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H52" s="20" t="str">
+        <x:v>/tmp/pptbridge_live_powerpoint_final + /tmp/pptbridge_live_start_final</x:v>
+      </x:c>
+      <x:c r="I52" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="64" customHeight="1">
+      <x:c r="A53" s="20" t="str">
+        <x:v>T-049</x:v>
+      </x:c>
+      <x:c r="B53" s="20" t="str">
+        <x:v>ROUTE-001/LIVE-001</x:v>
+      </x:c>
+      <x:c r="C53" s="20" t="str">
+        <x:v>Independent multi-live sessions</x:v>
+      </x:c>
+      <x:c r="D53" s="20" t="str">
+        <x:v>Start and navigate two different PowerPoint decks concurrently.</x:v>
+      </x:c>
+      <x:c r="E53" s="20" t="str">
+        <x:v>Each source owns the correct session and navigation does not affect the other deck.</x:v>
+      </x:c>
+      <x:c r="F53" s="20" t="str">
+        <x:v>Two distinct live decks opened through LaunchServices, started in separate windows, navigated independently, and stopped cleanly.</x:v>
+      </x:c>
+      <x:c r="G53" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H53" s="20" t="str">
+        <x:v>/tmp/pptbridge_multi_live_smoke_v058_launchservices on 2026-07-18</x:v>
+      </x:c>
+      <x:c r="I53" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="64" customHeight="1">
+      <x:c r="A54" s="20" t="str">
+        <x:v>T-050</x:v>
+      </x:c>
+      <x:c r="B54" s="20" t="str">
+        <x:v>SRC-001/SRC-002/ROUTE-001/PRES-001/LIVE-007</x:v>
+      </x:c>
+      <x:c r="C54" s="20" t="str">
+        <x:v>Real OBS visual WebSocket smoke</x:v>
+      </x:c>
+      <x:c r="D54" s="20" t="str">
+        <x:v>Create PPTX/PDF slide and presenter sources in OBS 32.1.1 Studio Mode, route two decks, customize presenter view, exercise live/final/black/stop, and capture screenshots.</x:v>
+      </x:c>
+      <x:c r="E54" s="20" t="str">
+        <x:v>Outputs are nonblank and correctly framed; Program routing, presenter layout, final guard, black, and PDF navigation work.</x:v>
+      </x:c>
+      <x:c r="F54" s="20" t="str">
+        <x:v>Final installed-plugin run passed every reported state, including focused hotkeys, source/property buttons, two-scene routing, Presenter customization, cue checks, all 16 OSC feedback paths, manual/auto live start-stop, reattach, final-slide guard, and black restore.</x:v>
+      </x:c>
+      <x:c r="G54" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H54" s="20" t="str">
+        <x:v>qa/obs-websocket-smoke.mjs; /tmp/pptbridge-v058-final-runtime-14</x:v>
+      </x:c>
+      <x:c r="I54" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="64" customHeight="1">
+      <x:c r="A55" s="20" t="str">
+        <x:v>T-051</x:v>
+      </x:c>
+      <x:c r="B55" s="20" t="str">
+        <x:v>NAV-001/CUE-001/CUE-003</x:v>
+      </x:c>
+      <x:c r="C55" s="20" t="str">
+        <x:v>Installed OBS property status refresh</x:v>
+      </x:c>
+      <x:c r="D55" s="20" t="str">
+        <x:v>Use Next, Check Current Cue, and Clear Cue Checks in the real source properties dialog.</x:v>
+      </x:c>
+      <x:c r="E55" s="20" t="str">
+        <x:v>Operator and Source status panels update immediately and remain consistent.</x:v>
+      </x:c>
+      <x:c r="F55" s="20" t="str">
+        <x:v>Both panels changed to slide 2, showed checked count 1, then reset to zero.</x:v>
+      </x:c>
+      <x:c r="G55" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H55" s="20" t="str">
+        <x:v>Manual Computer Use test in installed OBS on 2026-07-15</x:v>
+      </x:c>
+      <x:c r="I55" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="64" customHeight="1">
+      <x:c r="A56" s="20" t="str">
+        <x:v>T-052</x:v>
+      </x:c>
+      <x:c r="B56" s="20" t="str">
+        <x:v>MEDIA-001/AUDIO-001/AUDIO-003</x:v>
+      </x:c>
+      <x:c r="C56" s="20" t="str">
+        <x:v>Embedded WAV/MP3 audio runtime</x:v>
+      </x:c>
+      <x:c r="D56" s="20" t="str">
+        <x:v>Load synthetic WAV and MP3 PPTX fixtures in installed OBS, inspect parent meter, and record output.</x:v>
+      </x:c>
+      <x:c r="E56" s="20" t="str">
+        <x:v>Parent source meter and recording contain one correctly leveled audio stream.</x:v>
+      </x:c>
+      <x:c r="F56" s="20" t="str">
+        <x:v>WAV and MP3 both populated the parent meter and recordings; unity max was -21.3 dB with no +6 dB duplication.</x:v>
+      </x:c>
+      <x:c r="G56" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H56" s="20" t="str">
+        <x:v>qa/obs-audio-runtime-smoke.mjs + recording analysis</x:v>
+      </x:c>
+      <x:c r="I56" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="64" customHeight="1">
+      <x:c r="A57" s="20" t="str">
+        <x:v>T-053</x:v>
+      </x:c>
+      <x:c r="B57" s="20" t="str">
+        <x:v>AUDIO-001/AUDIO-003</x:v>
+      </x:c>
+      <x:c r="C57" s="20" t="str">
+        <x:v>Audio gain and disable controls</x:v>
+      </x:c>
+      <x:c r="D57" s="20" t="str">
+        <x:v>Compare unity, -20 dB, and disabled audio runs.</x:v>
+      </x:c>
+      <x:c r="E57" s="20" t="str">
+        <x:v>Gain change is exact and disabled output is silent.</x:v>
+      </x:c>
+      <x:c r="F57" s="20" t="str">
+        <x:v>-20 dB produced an exact 20 dB reduction; disabled output was silent.</x:v>
+      </x:c>
+      <x:c r="G57" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H57" s="20" t="str">
+        <x:v>OBS audio runtime recordings on 2026-07-15</x:v>
+      </x:c>
+      <x:c r="I57" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="64" customHeight="1">
+      <x:c r="A58" s="20" t="str">
+        <x:v>T-054</x:v>
+      </x:c>
+      <x:c r="B58" s="20" t="str">
+        <x:v>MEDIA-001/AUDIO-001</x:v>
+      </x:c>
+      <x:c r="C58" s="20" t="str">
+        <x:v>Audio lifecycle stress</x:v>
+      </x:c>
+      <x:c r="D58" s="20" t="str">
+        <x:v>Create/destroy media-backed sources more than 120 times and monitor RSS over the second 50-cycle window.</x:v>
+      </x:c>
+      <x:c r="E58" s="20" t="str">
+        <x:v>No callback use-after-free, crash, or unbounded memory growth occurs.</x:v>
+      </x:c>
+      <x:c r="F58" s="20" t="str">
+        <x:v>120+ cycles passed; RSS increased only 0.2 MB across the second 50 cycles.</x:v>
+      </x:c>
+      <x:c r="G58" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H58" s="20" t="str">
+        <x:v>qa/obs-audio-runtime-smoke.mjs stress run</x:v>
+      </x:c>
+      <x:c r="I58" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="64" customHeight="1">
+      <x:c r="A59" s="20" t="str">
+        <x:v>T-055</x:v>
+      </x:c>
+      <x:c r="B59" s="20" t="str">
+        <x:v>LIVE-005/MEDIA-001</x:v>
+      </x:c>
+      <x:c r="C59" s="20" t="str">
+        <x:v>Shutdown during active audio</x:v>
+      </x:c>
+      <x:c r="D59" s="20" t="str">
+        <x:v>Quit OBS while embedded audio is active, inspect crash reports, then cold-start and retest audio.</x:v>
+      </x:c>
+      <x:c r="E59" s="20" t="str">
+        <x:v>OBS exits without PPTBridge crash and audio works after restart.</x:v>
+      </x:c>
+      <x:c r="F59" s="20" t="str">
+        <x:v>No new PPTBridge crash report; cold restart audio passed.</x:v>
+      </x:c>
+      <x:c r="G59" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H59" s="20" t="str">
+        <x:v>OBS logs and crash-report scan on 2026-07-15</x:v>
+      </x:c>
+      <x:c r="I59" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="64" customHeight="1">
+      <x:c r="A60" s="20" t="str">
+        <x:v>T-056</x:v>
+      </x:c>
+      <x:c r="B60" s="20" t="str">
+        <x:v>QA-001</x:v>
+      </x:c>
+      <x:c r="C60" s="20" t="str">
+        <x:v>ASan and UBSan regression suite</x:v>
+      </x:c>
+      <x:c r="D60" s="20" t="str">
+        <x:v>Run invalid input, registry, OSC command/feedback, and 15-deck render tests with sanitizers.</x:v>
+      </x:c>
+      <x:c r="E60" s="20" t="str">
+        <x:v>No memory-safety or undefined-behavior diagnostic is emitted.</x:v>
+      </x:c>
+      <x:c r="F60" s="20" t="str">
+        <x:v>All sanitizer tests passed; leak detection omitted because macOS ASan does not support it.</x:v>
+      </x:c>
+      <x:c r="G60" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H60" s="20" t="str">
+        <x:v>ASAN_OPTIONS=detect_leaks=0:halt_on_error=1; UBSAN_OPTIONS=halt_on_error=1</x:v>
+      </x:c>
+      <x:c r="I60" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="64" customHeight="1">
+      <x:c r="A61" s="20" t="str">
+        <x:v>T-057</x:v>
+      </x:c>
+      <x:c r="B61" s="20" t="str">
+        <x:v>QA-001</x:v>
+      </x:c>
+      <x:c r="C61" s="20" t="str">
+        <x:v>Clang static analyzer</x:v>
+      </x:c>
+      <x:c r="D61" s="20" t="str">
+        <x:v>Run Apple Clang --analyze using the six production compile commands.</x:v>
+      </x:c>
+      <x:c r="E61" s="20" t="str">
+        <x:v>Analyzer completes every production translation unit without diagnostics.</x:v>
+      </x:c>
+      <x:c r="F61" s="20" t="str">
+        <x:v>6/6 production files passed.</x:v>
+      </x:c>
+      <x:c r="G61" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H61" s="20" t="str">
+        <x:v>native-plugin/build/compile_commands.json analyzer run</x:v>
+      </x:c>
+      <x:c r="I61" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="64" customHeight="1">
+      <x:c r="A62" s="20" t="str">
+        <x:v>T-058</x:v>
+      </x:c>
+      <x:c r="B62" s="20" t="str">
+        <x:v>INSTALL-004/PACK-001</x:v>
+      </x:c>
+      <x:c r="C62" s="20" t="str">
+        <x:v>Release package dry run</x:v>
+      </x:c>
+      <x:c r="D62" s="20" t="str">
+        <x:v>Build the release staging tree and inspect ZIP members, architecture, signatures, junk, and duplicate paths.</x:v>
+      </x:c>
+      <x:c r="E62" s="20" t="str">
+        <x:v>Package contains only documented user files and arm64 signed plugin content.</x:v>
+      </x:c>
+      <x:c r="F62" s="20" t="str">
+        <x:v>20 entries, no duplicates or junk; plugin executable arm64 and ad-hoc signature valid.</x:v>
+      </x:c>
+      <x:c r="G62" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H62" s="20" t="str">
+        <x:v>native-plugin/scripts/make-release.sh dry run before version bump</x:v>
+      </x:c>
+      <x:c r="I62" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="64" customHeight="1">
+      <x:c r="A63" s="20" t="str">
+        <x:v>T-059</x:v>
+      </x:c>
+      <x:c r="B63" s="20" t="str">
+        <x:v>INSTALL-001</x:v>
+      </x:c>
+      <x:c r="C63" s="20" t="str">
+        <x:v>Isolated installer smoke</x:v>
+      </x:c>
+      <x:c r="D63" s="20" t="str">
+        <x:v>Run the packaged installer against an isolated test HOME with OBS closed.</x:v>
+      </x:c>
+      <x:c r="E63" s="20" t="str">
+        <x:v>Installer copies the plugin to the expected user plugin path and rejects unsafe install while OBS is open.</x:v>
+      </x:c>
+      <x:c r="F63" s="20" t="str">
+        <x:v>Isolated install succeeded; OBS-open safety refusal also passed.</x:v>
+      </x:c>
+      <x:c r="G63" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H63" s="20" t="str">
+        <x:v>packaged 1-Install-PPTBridge-SK.command isolated HOME test</x:v>
+      </x:c>
+      <x:c r="I63" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="64" customHeight="1">
+      <x:c r="A64" s="20" t="str">
+        <x:v>T-060</x:v>
+      </x:c>
+      <x:c r="B64" s="20" t="str">
+        <x:v>HOTKEY-001/HOTKEY-002/HOTKEY-003/HOTKEY-004</x:v>
+      </x:c>
+      <x:c r="C64" s="20" t="str">
+        <x:v>Installed OBS hotkey and keyboard focus matrix</x:v>
+      </x:c>
+      <x:c r="D64" s="20" t="str">
+        <x:v>Run official Next/Previous hotkey callbacks with OBS frontmost, repeat with another app/UI field active, and test plain Left/Right editing.</x:v>
+      </x:c>
+      <x:c r="E64" s="20" t="str">
+        <x:v>Focused callbacks navigate and restore the Program deck; out-of-focus callbacks and plain arrows leave the deck unchanged.</x:v>
+      </x:c>
+      <x:c r="F64" s="20" t="str">
+        <x:v>Next changed the source, Previous restored it, out-of-focus guard ignored normal input, and ABCDXEY cursor-edit test passed.</x:v>
+      </x:c>
+      <x:c r="G64" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H64" s="20" t="str">
+        <x:v>qa/obs-websocket-smoke.mjs plus hands-on OBS field test on 2026-07-16</x:v>
+      </x:c>
+      <x:c r="I64" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="64" customHeight="1">
+      <x:c r="A65" s="20" t="str">
+        <x:v>T-061</x:v>
+      </x:c>
+      <x:c r="B65" s="20" t="str">
+        <x:v>OSCFB-001/OSCFB-002/OSCFB-003/OSCFB-004</x:v>
+      </x:c>
+      <x:c r="C65" s="20" t="str">
+        <x:v>Installed OBS OSC feedback runtime</x:v>
+      </x:c>
+      <x:c r="D65" s="20" t="str">
+        <x:v>Enable feedback in the installed source, listen on UDP 57131, navigate, check cues, and validate every documented field.</x:v>
+      </x:c>
+      <x:c r="E65" s="20" t="str">
+        <x:v>All 16 feedback addresses carry accurate current source/deck/slide/live/loading/error/timer/cue state.</x:v>
+      </x:c>
+      <x:c r="F65" s="20" t="str">
+        <x:v>16/16 fields passed against PPTBridge QA Slide A with accurate current/total/title/next/deck/source/error/timer/live/loading/loaded/black/cue values.</x:v>
+      </x:c>
+      <x:c r="G65" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H65" s="20" t="str">
+        <x:v>qa/obs-feedback-runtime-smoke.mjs on 2026-07-16</x:v>
+      </x:c>
+      <x:c r="I65" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="64" customHeight="1">
+      <x:c r="A66" s="20" t="str">
+        <x:v>T-062</x:v>
+      </x:c>
+      <x:c r="B66" s="20" t="str">
+        <x:v>COMP-001/LIVE-001/LIVE-003/NAV-001/LIVE-007</x:v>
+      </x:c>
+      <x:c r="C66" s="20" t="str">
+        <x:v>Companion property-button runtime</x:v>
+      </x:c>
+      <x:c r="D66" s="20" t="str">
+        <x:v>Use authenticated OBS WebSocket PressInputPropertiesButton for Next, Previous, Start Live, Stop Live, and Restart on an installed source.</x:v>
+      </x:c>
+      <x:c r="E66" s="20" t="str">
+        <x:v>Each documented property button changes the expected rendered state and returns cleanly; Restart works after explicit Stop and Next at the final slide keeps the output open.</x:v>
+      </x:c>
+      <x:c r="F66" s="20" t="str">
+        <x:v>Installed OBS run passed Next, Previous, manual Start, Stop, Restart, reattach, final-slide guard, and explicit return to static output.</x:v>
+      </x:c>
+      <x:c r="G66" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H66" s="20" t="str">
+        <x:v>qa/obs-websocket-smoke.mjs on 2026-07-18</x:v>
+      </x:c>
+      <x:c r="I66" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="64" customHeight="1">
+      <x:c r="A67" s="20" t="str">
+        <x:v>T-063</x:v>
+      </x:c>
+      <x:c r="B67" s="20" t="str">
+        <x:v>INSTALL-001/INSTALL-004/PACK-001</x:v>
+      </x:c>
+      <x:c r="C67" s="20" t="str">
+        <x:v>Exact v0.5.8 package and installer</x:v>
+      </x:c>
+      <x:c r="D67" s="20" t="str">
+        <x:v>Create the ZIP twice, compare extracted trees, inspect entries/architecture/signature, verify SHA, and install the exact packaged bundle in isolated and real user paths.</x:v>
+      </x:c>
+      <x:c r="E67" s="20" t="str">
+        <x:v>Packaging is deterministic, minimal, arm64, installable, and its checksum matches.</x:v>
+      </x:c>
+      <x:c r="F67" s="20" t="str">
+        <x:v>Two frozen package runs produced the identical SHA-256 72ff22a6e6b895d81ce19c7bc40fa4722dc68cf62825a4f16fe455c703664719. The ZIP has 20 expected entries with no duplicate/junk paths; its arm64 0.5.8 plugin signature and checksum passed, and its exact installer copied an identical executable into an isolated HOME.</x:v>
+      </x:c>
+      <x:c r="G67" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H67" s="20" t="str">
+        <x:v>native-plugin/scripts/make-release.sh; /tmp/pptbridge-v058-exact-final</x:v>
+      </x:c>
+      <x:c r="I67" s="20" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="64" customHeight="1">
+      <x:c r="A68" s="20" t="str">
+        <x:v>T-064</x:v>
+      </x:c>
+      <x:c r="B68" s="20" t="str">
+        <x:v>LIVE-005/QA-001</x:v>
+      </x:c>
+      <x:c r="C68" s="20" t="str">
+        <x:v>Graceful shutdown and environment restoration</x:v>
+      </x:c>
+      <x:c r="D68" s="20" t="str">
+        <x:v>Quit installed OBS during an owned live PowerPoint session, inspect logs/crash reports/processes, remove QA scenes, and restore OBS configs from byte-exact backups.</x:v>
+      </x:c>
+      <x:c r="E68" s="20" t="str">
+        <x:v>Live slideshow and OSC stop, OBS exits without a new PPTBridge crash, QA objects disappear, and user configs match backups.</x:v>
+      </x:c>
+      <x:c r="F68" s="20" t="str">
+        <x:v>Final QA cleanup removed its scenes and sources; WebSocket config and global.ini were restored byte-for-byte with their saved SHA-256 values.</x:v>
+      </x:c>
+      <x:c r="G68" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H68" s="20" t="str">
+        <x:v>OBS runtime-14 cleanup and SHA-256 verification on 2026-07-18</x:v>
+      </x:c>
+      <x:c r="I68" s="20" t="str">
+        <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4806,13 +5599,13 @@
     <x:mergeCell ref="A2:N2"/>
   </x:mergeCells>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="G5:G43">
+    <x:dataValidation type="list" sqref="G5:G68">
       <x:formula1>"Pass,Fail,Not Run,Blocked,Retest Required"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d21c7e3830a426a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re303c10296e44faa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4915,7 +5708,7 @@
         <x:v>HOTKEY-004</x:v>
       </x:c>
       <x:c r="C6" s="20" t="str">
-        <x:v>Open</x:v>
+        <x:v>Closed</x:v>
       </x:c>
       <x:c r="D6" s="20" t="str">
         <x:v>P0</x:v>
@@ -4927,16 +5720,16 @@
         <x:v>User reported left/right arrows unusable while OBS is open.</x:v>
       </x:c>
       <x:c r="G6" s="20" t="str">
-        <x:v>User report in thread</x:v>
+        <x:v>User report plus installed OBS field test</x:v>
       </x:c>
       <x:c r="H6" s="20" t="str">
-        <x:v>Do a hands-on OBS UI/text-field arrow-key check with clicker capture both off and on.</x:v>
+        <x:v>Keep the focused text-field and screenshot-state check in release regression.</x:v>
       </x:c>
       <x:c r="I6" s="20" t="str">
-        <x:v>Code/config audit is clean: PPTBridge hotkeys are 2/1 only and clicker capture filters plain left/right arrows. Automated GUI harness could not acquire normal frontmost focus from Codex.</x:v>
+        <x:v>Defaults remain 2/1, clicker capture filters plain arrows, and the installed OBS ABCDXEY cursor-edit test proved Left/Right are delivered normally without navigating slides.</x:v>
       </x:c>
       <x:c r="J6" s="20" t="str">
-        <x:v>Code/config pass; manual UI retest still required</x:v>
+        <x:v>Retested Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="72" customHeight="1">
@@ -4968,6 +5761,102 @@
         <x:v>AppleScript runner now keeps task output as std::string, idle PowerPoint retry parsing uses stable comma output, fresh plugin-owned bad PowerPoint launches can be terminated for retry, and live start opens the original selected deck path before staged fallback.</x:v>
       </x:c>
       <x:c r="J7" s="20" t="str">
+        <x:v>Retested Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="72" customHeight="1">
+      <x:c r="A8" s="20" t="str">
+        <x:v>ISS-004</x:v>
+      </x:c>
+      <x:c r="B8" s="20" t="str">
+        <x:v>NAV-001/CUE-001/CUE-003</x:v>
+      </x:c>
+      <x:c r="C8" s="20" t="str">
+        <x:v>Closed</x:v>
+      </x:c>
+      <x:c r="D8" s="20" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="E8" s="20" t="str">
+        <x:v>Operator UX</x:v>
+      </x:c>
+      <x:c r="F8" s="20" t="str">
+        <x:v>Operator status refreshed after property buttons, but the lower Source status panel could remain stale until the dialog reopened.</x:v>
+      </x:c>
+      <x:c r="G8" s="20" t="str">
+        <x:v>Manual installed-OBS properties test on 2026-07-15</x:v>
+      </x:c>
+      <x:c r="H8" s="20" t="str">
+        <x:v>Keep the real properties-button status synchronization in release regression.</x:v>
+      </x:c>
+      <x:c r="I8" s="20" t="str">
+        <x:v>refresh_operator_status_property now refreshes both pptbridge_operator_status and pptbridge_status from the same document snapshot.</x:v>
+      </x:c>
+      <x:c r="J8" s="20" t="str">
+        <x:v>Retested Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="72" customHeight="1">
+      <x:c r="A9" s="20" t="str">
+        <x:v>ISS-005</x:v>
+      </x:c>
+      <x:c r="B9" s="20" t="str">
+        <x:v>MEDIA-001/AUDIO-001</x:v>
+      </x:c>
+      <x:c r="C9" s="20" t="str">
+        <x:v>Closed</x:v>
+      </x:c>
+      <x:c r="D9" s="20" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E9" s="20" t="str">
+        <x:v>Audio Routing</x:v>
+      </x:c>
+      <x:c r="F9" s="20" t="str">
+        <x:v>Embedded FFmpeg child media played but did not reliably populate the parent PPTBridge source meter or recording path.</x:v>
+      </x:c>
+      <x:c r="G9" s="20" t="str">
+        <x:v>Synthetic WAV/MP3 fixtures and OBS runtime recordings</x:v>
+      </x:c>
+      <x:c r="H9" s="20" t="str">
+        <x:v>Retain parent-meter, gain, disable, lifecycle, and shutdown audio tests before releases.</x:v>
+      </x:c>
+      <x:c r="I9" s="20" t="str">
+        <x:v>Child PCM is forwarded once to the parent source via obs_source_output_audio with balanced callback registration/removal; media lifecycle uses restart_on_activate and close_when_inactive=false.</x:v>
+      </x:c>
+      <x:c r="J9" s="20" t="str">
+        <x:v>Retested Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="72" customHeight="1">
+      <x:c r="A10" s="20" t="str">
+        <x:v>ISS-006</x:v>
+      </x:c>
+      <x:c r="B10" s="20" t="str">
+        <x:v>LOAD-004</x:v>
+      </x:c>
+      <x:c r="C10" s="20" t="str">
+        <x:v>Closed</x:v>
+      </x:c>
+      <x:c r="D10" s="20" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="E10" s="20" t="str">
+        <x:v>Input Validation</x:v>
+      </x:c>
+      <x:c r="F10" s="20" t="str">
+        <x:v>Unsupported, corrupt, or missing presentation paths could enter the loader before a precise user-facing rejection.</x:v>
+      </x:c>
+      <x:c r="G10" s="20" t="str">
+        <x:v>Sanitizer invalid-input smoke</x:v>
+      </x:c>
+      <x:c r="H10" s="20" t="str">
+        <x:v>Keep corrupt PPTX/PDF and missing-file cases in automated regression.</x:v>
+      </x:c>
+      <x:c r="I10" s="20" t="str">
+        <x:v>Strict extension/existence/ZIP/PDFKit validation now rejects invalid input with actionable errors before loading.</x:v>
+      </x:c>
+      <x:c r="J10" s="20" t="str">
         <x:v>Retested Pass</x:v>
       </x:c>
     </x:row>
@@ -4977,16 +5866,16 @@
     <x:mergeCell ref="A2:N2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C5:C7">
+    <x:dataValidation type="list" sqref="C5:C10">
       <x:formula1>"Open,Fixed,Retesting,Closed,Deferred"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D5:D7">
+    <x:dataValidation type="list" sqref="D5:D10">
       <x:formula1>"P0,P1,P2,P3"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9acef69480a44d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R886a0d676c344ef1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Release Apple Silicon v0.5.11
</commit_message>
<xml_diff>
--- a/qa/PPTBridge-Feature-QA-Tracker.xlsx
+++ b/qa/PPTBridge-Feature-QA-Tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R43e4cce1276549d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UserStories" sheetId="2" r:id="Rff047d0e44214fb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestLog" sheetId="3" r:id="Ra782aa685bdf4785"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issues" sheetId="4" r:id="R5d100647fd864499"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R8ec773b3b15d4f5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UserStories" sheetId="2" r:id="R79341bb43e0b4f7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestLog" sheetId="3" r:id="Rd0248c0f9726443a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issues" sheetId="4" r:id="Re6a69b2595fe4888"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TestLogTable" displayName="TestLogTable" ref="A4:I68" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TestLogTable" displayName="TestLogTable" ref="A4:I79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Story ID"/>
@@ -206,7 +206,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="IssuesTable" displayName="IssuesTable" ref="A4:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="IssuesTable" displayName="IssuesTable" ref="A4:J11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Issue ID"/>
     <x:tableColumn id="2" name="Story ID"/>
@@ -435,7 +435,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="5" t="str">
-        <x:v>Single canonical tracker for feature coverage, user stories, testing, issues, and retesting. Generated 2026-07-18.</x:v>
+        <x:v>Single canonical tracker for feature coverage, user stories, testing, issues, and retesting. Generated 2026-08-25.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -460,7 +460,7 @@
       </x:c>
       <x:c r="B6" s="14" t="n">
         <x:f>COUNTIF('UserStories'!J5:J74,"Verified")+COUNTIF('UserStories'!J5:J74,"Pass")</x:f>
-        <x:v>53</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -469,7 +469,7 @@
       </x:c>
       <x:c r="B7" s="14" t="n">
         <x:f>COUNTIF('UserStories'!J5:J74,"Needs Manual")</x:f>
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -478,7 +478,7 @@
       </x:c>
       <x:c r="B8" s="14" t="n">
         <x:f>COUNTIF('UserStories'!J5:J74,"Not Run")</x:f>
-        <x:v>9</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -495,7 +495,7 @@
         <x:v>Open issues</x:v>
       </x:c>
       <x:c r="B10" s="14" t="n">
-        <x:f>COUNTIF('Issues'!C5:C10,"Open")</x:f>
+        <x:f>COUNTIF('Issues'!C5:C11,"Open")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -513,7 +513,7 @@
         <x:v>Release state</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>v0.5.8 stable package verified and ready for publication</x:v>
+        <x:v>v0.5.11 Apple Silicon stable package verified; Windows remains v0.5.10 beta</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -567,7 +567,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="5" t="str">
-        <x:v>Canonical user-story tracker generated 2026-07-18. Source repo: https://github.com/srdjankotarlic/pptbridge-sk-obs</x:v>
+        <x:v>Canonical user-story tracker generated 2026-08-25. Source repo: https://github.com/srdjankotarlic/pptbridge-sk-obs</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -652,7 +652,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M5" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N5" s="20" t="str">
         <x:v>2026-07-15 real OBS WebSocket smoke added Slide sources for PPTX/PDF, rendered nonblank 1920x1080 output, and captured screenshots.</x:v>
@@ -696,7 +696,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M6" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N6" s="20" t="str">
         <x:v>2026-07-15 real OBS smoke rendered current/next slides, notes, timer, cue list, and customized presenter layouts.</x:v>
@@ -740,7 +740,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M7" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N7" s="20" t="str">
         <x:v>2026-07-15 13 real PPTX/PDF decks plus two media fixtures passed render and navigation; real OBS source selection passed.</x:v>
@@ -784,7 +784,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M8" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N8" s="20" t="str">
         <x:v>2026-07-15 three real PDFs passed render/navigation and real OBS PDF screenshots showed correct first/next pages.</x:v>
@@ -828,7 +828,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M9" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N9" s="20" t="str">
         <x:v>Needs real Windows runtime test.</x:v>
@@ -872,7 +872,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M10" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N10" s="20" t="str">
         <x:v>2026-06-23 smoke: large uncached PPTX first preview 7668 ms; same deck cached preview 46 ms; small cached PPTX 47 ms; PDF 56 ms.</x:v>
@@ -916,7 +916,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M11" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N11" s="20" t="str">
         <x:v>2026-07-15 render matrix and installed OBS presenter source showed first preview before notes/cue preparation completed, then refreshed with notes and cue data.</x:v>
@@ -951,7 +951,7 @@
         <x:v>Button + OSC smoke</x:v>
       </x:c>
       <x:c r="J12" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K12" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -960,9 +960,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M12" s="20" t="str">
-        <x:v>2026-07-18</x:v>
-      </x:c>
-      <x:c r="N12" s="20" t="str"/>
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="N12" s="20" t="str">
+        <x:v>2026-08-25 real OBS WebSocket regression pressed Reload and confirmed the installed source returned a valid rendered deck.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
       <x:c r="A13" s="20" t="str">
@@ -1002,7 +1004,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M13" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N13" s="20" t="str">
         <x:v>2026-07-15 ASan/UBSan smoke rejected empty path, missing PPTX, wrong extension, corrupt PPTX, and corrupt PDF with explicit errors and no crash.</x:v>
@@ -1046,7 +1048,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M14" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N14" s="20" t="str">
         <x:v>2026-06-23 large PPTX reload reused cached PDF: PDF prep 0 ms, first preview 46 ms, full load 239 ms.</x:v>
@@ -1090,7 +1092,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M15" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N15" s="20" t="str">
         <x:v>2026-06-23 final smoke: original Desktop PPTX started live mode, advanced to slide 2, and stopped slideshow.</x:v>
@@ -1134,7 +1136,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M16" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N16" s="20" t="str">
         <x:v>2026-06-23 smoke covered both immediate StartLivePowerPointAsync and preview-first manual start.</x:v>
@@ -1178,7 +1180,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M17" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N17" s="20" t="str"/>
     </x:row>
@@ -1220,7 +1222,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M18" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N18" s="20" t="str">
         <x:v>2026-07-16 real OBS WebSocket smoke enabled auto-start on an existing source and captured a nonblank live PowerPoint frame.</x:v>
@@ -1264,7 +1266,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M19" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N19" s="20" t="str">
         <x:v>2026-07-15 two controlled OBS quit/restart cycles completed without a new PPTBridge crash report.</x:v>
@@ -1308,7 +1310,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M20" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N20" s="20" t="str">
         <x:v>2026-07-15 watchdog recovery restarted an externally closed healthy slideshow; explicit Stop remained stopped.</x:v>
@@ -1352,7 +1354,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M21" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N21" s="20" t="str">
         <x:v>2026-07-15 direct live smoke and real OBS screenshot-hash test both kept the final slide visible after repeated Next commands.</x:v>
@@ -1396,7 +1398,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M22" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N22" s="20" t="str">
         <x:v>v0.5.6 change; verify visually again.</x:v>
@@ -1440,7 +1442,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M23" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N23" s="20" t="str">
         <x:v>2026-06-23 temp and hidden sidecar staging reproduced PowerPoint hangs; final code uses original path first and passed live_start/live_powerpoint smokes on the original Desktop PPTX.</x:v>
@@ -1475,7 +1477,7 @@
         <x:v>Manual resize test</x:v>
       </x:c>
       <x:c r="J24" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K24" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -1484,9 +1486,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M24" s="20" t="str">
-        <x:v>2026-07-18</x:v>
-      </x:c>
-      <x:c r="N24" s="20" t="str"/>
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="N24" s="20" t="str">
+        <x:v>2026-08-25 real OBS runtime confirmed lock_canvas persists and keeps the OBS output dimensions stable.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="58" customHeight="1">
       <x:c r="A25" s="20" t="str">
@@ -1517,7 +1521,7 @@
         <x:v>Manual resize test</x:v>
       </x:c>
       <x:c r="J25" s="20" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K25" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -1526,9 +1530,11 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M25" s="20" t="str">
-        <x:v>2026-07-18</x:v>
-      </x:c>
-      <x:c r="N25" s="20" t="str"/>
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="N25" s="20" t="str">
+        <x:v>2026-08-25 real OBS runtime confirmed fit_window persists and can be switched back to lock_canvas.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="58" customHeight="1">
       <x:c r="A26" s="20" t="str">
@@ -1559,7 +1565,7 @@
         <x:v>Manual live recovery test</x:v>
       </x:c>
       <x:c r="J26" s="20" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K26" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -1568,9 +1574,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M26" s="20" t="str">
-        <x:v>2026-07-18</x:v>
-      </x:c>
-      <x:c r="N26" s="20" t="str"/>
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="N26" s="20" t="str">
+        <x:v>2026-08-25 installed OBS runtime reattached to the same live PowerPoint output and preserved the expected frame.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="58" customHeight="1">
       <x:c r="A27" s="20" t="str">
@@ -1610,7 +1618,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M27" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N27" s="20" t="str">
         <x:v>2026-07-15 manual installed-OBS properties test confirmed Next/Previous update both Operator and Source status immediately.</x:v>
@@ -1645,7 +1653,7 @@
         <x:v>OBS property button test</x:v>
       </x:c>
       <x:c r="J28" s="20" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K28" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -1654,9 +1662,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M28" s="20" t="str">
-        <x:v>2026-07-18</x:v>
-      </x:c>
-      <x:c r="N28" s="20" t="str"/>
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="N28" s="20" t="str">
+        <x:v>2026-08-25 standalone and real OBS runtime tests covered first/last navigation and final-slide protection.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">
       <x:c r="A29" s="20" t="str">
@@ -1696,7 +1706,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M29" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N29" s="20" t="str">
         <x:v>2026-07-15 real OBS visual smoke captured black output and confirmed the original slide restored after toggling back.</x:v>
@@ -1740,7 +1750,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M30" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N30" s="20" t="str">
         <x:v>2026-07-16 profile inspection confirmed only 2/1 defaults; installed OBS invoked the registered Next/Previous callbacks and restored the initial slide.</x:v>
@@ -1784,7 +1794,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M31" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N31" s="20" t="str">
         <x:v>2026-07-16 official TriggerHotkeyByName calls exercised the registered callbacks in frontmost OBS and changed only the Program-scene deck.</x:v>
@@ -1828,7 +1838,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M32" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N32" s="20" t="str">
         <x:v>2026-07-16 out-of-focus callback guard left the slide unchanged while normal text entry continued in another UI field.</x:v>
@@ -1872,7 +1882,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M33" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N33" s="20" t="str">
         <x:v>2026-07-16 hands-on installed OBS test typed ABCDE, moved Left, inserted X, moved Right, inserted Y, and produced ABCDXEY; the presentation stayed on slide 1 and plain Left/Right never triggered navigation.</x:v>
@@ -1907,7 +1917,7 @@
         <x:v>OBS menu + permissions test</x:v>
       </x:c>
       <x:c r="J34" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K34" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -1916,9 +1926,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M34" s="20" t="str">
-        <x:v>2026-07-18</x:v>
-      </x:c>
-      <x:c r="N34" s="20" t="str"/>
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="N34" s="20" t="str">
+        <x:v>2026-08-25 real macOS event-tap test confirmed enabled capture and safe disable behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="58" customHeight="1">
       <x:c r="A35" s="20" t="str">
@@ -1949,7 +1961,7 @@
         <x:v>Global keyboard/clicker test</x:v>
       </x:c>
       <x:c r="J35" s="20" t="str">
-        <x:v>Needs Manual</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K35" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -1958,9 +1970,11 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M35" s="20" t="str">
-        <x:v>2026-07-18</x:v>
-      </x:c>
-      <x:c r="N35" s="20" t="str"/>
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="N35" s="20" t="str">
+        <x:v>2026-08-25 PageDown/PageUp moved and restored only the Program deck while another app owned focus.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="58" customHeight="1">
       <x:c r="A36" s="20" t="str">
@@ -1991,7 +2005,7 @@
         <x:v>Global keyboard test</x:v>
       </x:c>
       <x:c r="J36" s="20" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="K36" s="20" t="str">
         <x:v>Implemented</x:v>
@@ -2000,9 +2014,11 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M36" s="20" t="str">
-        <x:v>2026-07-18</x:v>
-      </x:c>
-      <x:c r="N36" s="20" t="str"/>
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="N36" s="20" t="str">
+        <x:v>2026-08-25 key-receiver app confirmed PageDown/PageUp were suppressed while Left/Right/Space still reached the focused app.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="58" customHeight="1">
       <x:c r="A37" s="20" t="str">
@@ -2042,7 +2058,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M37" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N37" s="20" t="str"/>
     </x:row>
@@ -2084,7 +2100,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M38" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N38" s="20" t="str">
         <x:v>2026-07-15 real OBS Studio Mode test: deck A changed while B stayed stable; after Program switched to B, only B changed. Preview never stole routing.</x:v>
@@ -2128,7 +2144,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M39" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N39" s="20" t="str"/>
     </x:row>
@@ -2170,7 +2186,7 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="M40" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N40" s="20" t="str">
         <x:v>Windows intentionally requires Program scene.</x:v>
@@ -2214,7 +2230,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M41" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N41" s="20" t="str">
         <x:v>2026-07-16 installed OBS bound 127.0.0.1:57130, accepted runtime commands, and logged a clean listener shutdown.</x:v>
@@ -2258,7 +2274,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M42" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N42" s="20" t="str">
         <x:v>2026-07-15 ASan/UBSan OSC smoke passed all 8 supported command paths and ignored malformed/unknown packets.</x:v>
@@ -2302,7 +2318,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M43" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N43" s="20" t="str">
         <x:v>2026-07-16 real OBS Studio Mode smoke sent OSC Next with deck A then deck B in Program; only the current Program deck changed and Preview never stole routing.</x:v>
@@ -2346,7 +2362,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M44" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N44" s="20" t="str">
         <x:v>2026-07-15 real installed-OBS feedback receiver and isolated sender smoke both passed.</x:v>
@@ -2390,7 +2406,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M45" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N45" s="20" t="str">
         <x:v>2026-07-15 all 16 feedback fields passed with accurate slide/title state after navigation.</x:v>
@@ -2434,7 +2450,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M46" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N46" s="20" t="str">
         <x:v>2026-07-15 runtime feedback smoke verified deck/file/source/loading/loaded/error/timer/live/black fields.</x:v>
@@ -2478,7 +2494,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M47" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N47" s="20" t="str">
         <x:v>2026-07-15 manual cue check/clear in installed OBS plus 16-field feedback smoke verified current/next/checked count.</x:v>
@@ -2522,7 +2538,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M48" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N48" s="20" t="str">
         <x:v>2026-07-16 installed OBS smoke used PressInputPropertiesButton for Previous, Next, Start Live, and Stop Live and verified each rendered state.</x:v>
@@ -2566,7 +2582,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M49" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N49" s="20" t="str"/>
     </x:row>
@@ -2608,7 +2624,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M50" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N50" s="20" t="str">
         <x:v>2026-07-15 render matrix exercised all presets and real OBS visual smoke confirmed balanced and large-notes layouts.</x:v>
@@ -2652,7 +2668,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M51" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N51" s="20" t="str">
         <x:v>2026-07-15 sanitizer render matrix covered fit/fill/crop and position variants; installed OBS customization changed only the Presenter screenshot.</x:v>
@@ -2696,7 +2712,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M52" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N52" s="20" t="str">
         <x:v>2026-07-15 installed OBS large-notes layout with 24 pt/130% notes changed the output; screenshots were inspected for clipping and overlap.</x:v>
@@ -2740,7 +2756,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M53" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N53" s="20" t="str">
         <x:v>2026-07-15 background image/mode/opacity smoke passed without obscuring presenter content.</x:v>
@@ -2784,7 +2800,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M54" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N54" s="20" t="str">
         <x:v>2026-07-15 render matrix and real OBS screenshots verified next-slide updates and the final End / No next slide state.</x:v>
@@ -2828,7 +2844,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M55" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N55" s="20" t="str">
         <x:v>2026-07-15 real OBS presenter screenshot visually confirmed cue list, current/next state, and checked cue changes.</x:v>
@@ -2872,7 +2888,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M56" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N56" s="20" t="str">
         <x:v>2026-07-15 installed-OBS button test updated both status panels and checked count; OSC state smoke passed.</x:v>
@@ -2916,7 +2932,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M57" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N57" s="20" t="str">
         <x:v>2026-07-16 installed OBS button sequence produced checked counts 1 then 2; render smoke also verified the no-next edge is ignored safely.</x:v>
@@ -2960,7 +2976,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M58" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N58" s="20" t="str">
         <x:v>2026-07-15 installed-OBS Clear Cue Checks button reset checked count to zero and refreshed both status panels.</x:v>
@@ -3004,7 +3020,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M59" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N59" s="20" t="str">
         <x:v>2026-07-15 cue export smoke produced readable slide/cue text and reported the output path.</x:v>
@@ -3048,7 +3064,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M60" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N60" s="20" t="str">
         <x:v>2026-07-15 synthetic WAV and MP3 PPTX fixtures created FFmpeg child media, populated the parent OBS meter, and recorded audible PCM.</x:v>
@@ -3092,7 +3108,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M61" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N61" s="20" t="str">
         <x:v>2026-07-15 installed-OBS audio smoke confirmed enabled output and complete silence when disabled.</x:v>
@@ -3136,7 +3152,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M62" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N62" s="20" t="str"/>
     </x:row>
@@ -3178,7 +3194,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M63" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N63" s="20" t="str">
         <x:v>2026-07-15 -20 dB setting measured an exact 20 dB reduction; unity gain showed no duplicate +6 dB mix.</x:v>
@@ -3222,7 +3238,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="M64" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N64" s="20" t="str">
         <x:v>2026-07-16 exact v0.5.8 ZIP installer passed in isolated HOME and real user install; installed arm64 binary loaded in OBS 32.1.1.</x:v>
@@ -3266,7 +3282,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M65" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N65" s="20" t="str"/>
     </x:row>
@@ -3308,7 +3324,7 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="M66" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N66" s="20" t="str"/>
     </x:row>
@@ -3350,7 +3366,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M67" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N67" s="20" t="str">
         <x:v>2026-07-16 v0.5.8 ZIP has exactly 20 documented entries, no duplicate paths, no Finder/build junk, and two independent package runs produced byte-identical extracted trees.</x:v>
@@ -3394,7 +3410,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M68" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N68" s="20" t="str">
         <x:v>Final frozen ZIP SHA-256 is 72ff22a6e6b895d81ce19c7bc40fa4722dc68cf62825a4f16fe455c703664719; the adjacent checksum file verified successfully.</x:v>
@@ -3438,7 +3454,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M69" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N69" s="20" t="str">
         <x:v>2026-07-16 README, Quickstart, setup, FAQ, packaged docs, and GitHub Pages content all describe v0.5.8 controls and install flow consistently.</x:v>
@@ -3482,7 +3498,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M70" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N70" s="20" t="str">
         <x:v>2026-07-16 documentation audit confirmed installation, permission, source visibility, live-mode, OSC/Companion, logs, and issue-reporting guidance.</x:v>
@@ -3526,7 +3542,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M71" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N71" s="20" t="str">
         <x:v>Tracks the QA process itself, not an end-user plugin feature.</x:v>
@@ -3570,7 +3586,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M72" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N72" s="20" t="str">
         <x:v>Out of scope for Mac-only validation.</x:v>
@@ -3614,7 +3630,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="M73" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N73" s="20" t="str"/>
     </x:row>
@@ -3656,7 +3672,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="M74" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N74" s="20" t="str"/>
     </x:row>
@@ -3678,7 +3694,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4f9a5974841490f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce56561890104f46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3763,7 +3779,7 @@
         <x:v>v0.5.6 release notes / local test run</x:v>
       </x:c>
       <x:c r="I5" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="64" customHeight="1">
@@ -3792,7 +3808,7 @@
         <x:v>native-plugin/tests/live_powerpoint_smoke.mm</x:v>
       </x:c>
       <x:c r="I6" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="64" customHeight="1">
@@ -3821,7 +3837,7 @@
         <x:v>rg --files output</x:v>
       </x:c>
       <x:c r="I7" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="64" customHeight="1">
@@ -3850,7 +3866,7 @@
         <x:v>Installed OBS hands-on field and slide-state test on 2026-07-16</x:v>
       </x:c>
       <x:c r="I8" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="64" customHeight="1">
@@ -3879,7 +3895,7 @@
         <x:v>/tmp/pptbridge_render_smoke /tmp/pptbridge-uncached-livepath-test.pptx</x:v>
       </x:c>
       <x:c r="I9" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="64" customHeight="1">
@@ -3908,7 +3924,7 @@
         <x:v>./build.sh</x:v>
       </x:c>
       <x:c r="I10" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="64" customHeight="1">
@@ -3937,7 +3953,7 @@
         <x:v>/tmp/pptbridge_osc_feedback_test</x:v>
       </x:c>
       <x:c r="I11" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="64" customHeight="1">
@@ -3966,7 +3982,7 @@
         <x:v>/tmp/pptbridge_render_smoke Desktop/PPT ZA PROBU PDF</x:v>
       </x:c>
       <x:c r="I12" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="64" customHeight="1">
@@ -3995,7 +4011,7 @@
         <x:v>/tmp/pptbridge_render_smoke Desktop/PPT ZA PROBU PPTX</x:v>
       </x:c>
       <x:c r="I13" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="64" customHeight="1">
@@ -4024,7 +4040,7 @@
         <x:v>osascript tell application /Applications/Microsoft PowerPoint.app</x:v>
       </x:c>
       <x:c r="I14" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="64" customHeight="1">
@@ -4053,7 +4069,7 @@
         <x:v>/tmp/pptbridge_live_start_smoke /tmp/pptbridge-uncached-livepath-test.pptx</x:v>
       </x:c>
       <x:c r="I15" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="64" customHeight="1">
@@ -4082,7 +4098,7 @@
         <x:v>OBS log 2026-06-22 00-23-32.txt</x:v>
       </x:c>
       <x:c r="I16" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="64" customHeight="1">
@@ -4111,7 +4127,7 @@
         <x:v>./build.sh on 2026-06-22</x:v>
       </x:c>
       <x:c r="I17" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="64" customHeight="1">
@@ -4140,7 +4156,7 @@
         <x:v>audit_guardrails.py on 2026-06-22</x:v>
       </x:c>
       <x:c r="I18" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="64" customHeight="1">
@@ -4169,7 +4185,7 @@
         <x:v>/tmp/pptbridge_render_smoke IV -1 Ana Dimitrijevic.pdf</x:v>
       </x:c>
       <x:c r="I19" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="64" customHeight="1">
@@ -4198,7 +4214,7 @@
         <x:v>/tmp/pptbridge_render_smoke II-3 Aldin Skenderi.pptx</x:v>
       </x:c>
       <x:c r="I20" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="64" customHeight="1">
@@ -4227,7 +4243,7 @@
         <x:v>/tmp/pptbridge_render_smoke /tmp/pptbridge-uncached-livepath-test.pptx</x:v>
       </x:c>
       <x:c r="I21" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="64" customHeight="1">
@@ -4256,7 +4272,7 @@
         <x:v>/tmp/pptbridge_live_start_smoke /tmp/pptbridge-uncached-livepath-test.pptx</x:v>
       </x:c>
       <x:c r="I22" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="64" customHeight="1">
@@ -4285,7 +4301,7 @@
         <x:v>basic.ini + plugin-main.mm inspection</x:v>
       </x:c>
       <x:c r="I23" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="64" customHeight="1">
@@ -4314,7 +4330,7 @@
         <x:v>/tmp/pptbridge_osc_feedback_test on 2026-06-22</x:v>
       </x:c>
       <x:c r="I24" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="64" customHeight="1">
@@ -4343,7 +4359,7 @@
         <x:v>artifact-tool import + formula scan on 2026-06-22</x:v>
       </x:c>
       <x:c r="I25" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="64" customHeight="1">
@@ -4372,7 +4388,7 @@
         <x:v>Installed OBS UI field plus screenshot state on 2026-07-16</x:v>
       </x:c>
       <x:c r="I26" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="64" customHeight="1">
@@ -4401,7 +4417,7 @@
         <x:v>./build.sh on 2026-06-23</x:v>
       </x:c>
       <x:c r="I27" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="64" customHeight="1">
@@ -4430,7 +4446,7 @@
         <x:v>/usr/bin/python3 native-plugin/tests/audit_guardrails.py on 2026-06-23</x:v>
       </x:c>
       <x:c r="I28" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="64" customHeight="1">
@@ -4459,7 +4475,7 @@
         <x:v>/tmp/pptbridge_render_smoke IV -1 Ana Dimitrijevic.pdf on 2026-06-23</x:v>
       </x:c>
       <x:c r="I29" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="64" customHeight="1">
@@ -4488,7 +4504,7 @@
         <x:v>/tmp/pptbridge_render_smoke II-3 Aldin Skenderi.pptx on 2026-06-23</x:v>
       </x:c>
       <x:c r="I30" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="64" customHeight="1">
@@ -4517,7 +4533,7 @@
         <x:v>/tmp/pptbridge_render_smoke /tmp/pptbridge-large-qa-20260623.pptx</x:v>
       </x:c>
       <x:c r="I31" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="64" customHeight="1">
@@ -4546,7 +4562,7 @@
         <x:v>/tmp/pptbridge_render_smoke /tmp/pptbridge-large-qa-20260623.pptx second run</x:v>
       </x:c>
       <x:c r="I32" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="64" customHeight="1">
@@ -4575,7 +4591,7 @@
         <x:v>/tmp/pptbridge_live_start_smoke Desktop/PPT ZA PROBU/II-5 Bajric - HEMOPTIZE.pptx</x:v>
       </x:c>
       <x:c r="I33" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="64" customHeight="1">
@@ -4604,7 +4620,7 @@
         <x:v>/tmp/pptbridge_live_powerpoint_smoke Desktop/PPT ZA PROBU/II-5 Bajric - HEMOPTIZE.pptx</x:v>
       </x:c>
       <x:c r="I34" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="64" customHeight="1">
@@ -4633,7 +4649,7 @@
         <x:v>/tmp/pptbridge_osc_feedback_test on 2026-06-23</x:v>
       </x:c>
       <x:c r="I35" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="64" customHeight="1">
@@ -4662,7 +4678,7 @@
         <x:v>git diff --check on 2026-06-23</x:v>
       </x:c>
       <x:c r="I36" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="64" customHeight="1">
@@ -4691,7 +4707,7 @@
         <x:v>/tmp/pptbridge_render_smoke cue status checks on 2026-06-23</x:v>
       </x:c>
       <x:c r="I37" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="64" customHeight="1">
@@ -4720,7 +4736,7 @@
         <x:v>OBS log 2026-06-23 02-41-51.txt</x:v>
       </x:c>
       <x:c r="I38" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="64" customHeight="1">
@@ -4749,7 +4765,7 @@
         <x:v>native-plugin/release/pptbridge-obs-macos-apple-silicon.zip</x:v>
       </x:c>
       <x:c r="I39" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="64" customHeight="1">
@@ -4778,7 +4794,7 @@
         <x:v>OBS log 2026-06-23 02-41-51.txt</x:v>
       </x:c>
       <x:c r="I40" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="64" customHeight="1">
@@ -4807,7 +4823,7 @@
         <x:v>/tmp/pptbridge_render_smoke II-3 Aldin Skenderi.pptx on 2026-06-23</x:v>
       </x:c>
       <x:c r="I41" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="64" customHeight="1">
@@ -4836,7 +4852,7 @@
         <x:v>/tmp/pptbridge_live_start_smoke + /tmp/pptbridge_live_powerpoint_smoke on 2026-06-23</x:v>
       </x:c>
       <x:c r="I42" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="64" customHeight="1">
@@ -4865,7 +4881,7 @@
         <x:v>Final smoke pass on 2026-06-23</x:v>
       </x:c>
       <x:c r="I43" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="64" customHeight="1">
@@ -4894,7 +4910,7 @@
         <x:v>cmake --build native-plugin/build --config Release --parallel on 2026-07-15</x:v>
       </x:c>
       <x:c r="I44" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="64" customHeight="1">
@@ -4923,7 +4939,7 @@
         <x:v>native-plugin/tests/audit_guardrails.py + git diff --check</x:v>
       </x:c>
       <x:c r="I45" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="64" customHeight="1">
@@ -4952,7 +4968,7 @@
         <x:v>/tmp/pptbridge_invalid_final_asan</x:v>
       </x:c>
       <x:c r="I46" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="64" customHeight="1">
@@ -4981,7 +4997,7 @@
         <x:v>/tmp/pptbridge_registry_final_asan</x:v>
       </x:c>
       <x:c r="I47" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="64" customHeight="1">
@@ -5010,7 +5026,7 @@
         <x:v>/tmp/pptbridge_osc_control_final_asan</x:v>
       </x:c>
       <x:c r="I48" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="64" customHeight="1">
@@ -5039,7 +5055,7 @@
         <x:v>/tmp/pptbridge_osc_feedback_final_asan</x:v>
       </x:c>
       <x:c r="I49" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="64" customHeight="1">
@@ -5068,7 +5084,7 @@
         <x:v>/tmp/pptbridge_render_v058_asan_current matrix on 2026-07-15</x:v>
       </x:c>
       <x:c r="I50" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="64" customHeight="1">
@@ -5097,7 +5113,7 @@
         <x:v>render smoke timing and cache timestamp test</x:v>
       </x:c>
       <x:c r="I51" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="64" customHeight="1">
@@ -5126,7 +5142,7 @@
         <x:v>/tmp/pptbridge_live_powerpoint_final + /tmp/pptbridge_live_start_final</x:v>
       </x:c>
       <x:c r="I52" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="64" customHeight="1">
@@ -5155,7 +5171,7 @@
         <x:v>/tmp/pptbridge_multi_live_smoke_v058_launchservices on 2026-07-18</x:v>
       </x:c>
       <x:c r="I53" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="64" customHeight="1">
@@ -5184,7 +5200,7 @@
         <x:v>qa/obs-websocket-smoke.mjs; /tmp/pptbridge-v058-final-runtime-14</x:v>
       </x:c>
       <x:c r="I54" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="64" customHeight="1">
@@ -5213,7 +5229,7 @@
         <x:v>Manual Computer Use test in installed OBS on 2026-07-15</x:v>
       </x:c>
       <x:c r="I55" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="64" customHeight="1">
@@ -5242,7 +5258,7 @@
         <x:v>qa/obs-audio-runtime-smoke.mjs + recording analysis</x:v>
       </x:c>
       <x:c r="I56" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="64" customHeight="1">
@@ -5271,7 +5287,7 @@
         <x:v>OBS audio runtime recordings on 2026-07-15</x:v>
       </x:c>
       <x:c r="I57" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="64" customHeight="1">
@@ -5300,7 +5316,7 @@
         <x:v>qa/obs-audio-runtime-smoke.mjs stress run</x:v>
       </x:c>
       <x:c r="I58" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="64" customHeight="1">
@@ -5329,7 +5345,7 @@
         <x:v>OBS logs and crash-report scan on 2026-07-15</x:v>
       </x:c>
       <x:c r="I59" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="64" customHeight="1">
@@ -5358,7 +5374,7 @@
         <x:v>ASAN_OPTIONS=detect_leaks=0:halt_on_error=1; UBSAN_OPTIONS=halt_on_error=1</x:v>
       </x:c>
       <x:c r="I60" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="64" customHeight="1">
@@ -5387,7 +5403,7 @@
         <x:v>native-plugin/build/compile_commands.json analyzer run</x:v>
       </x:c>
       <x:c r="I61" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="64" customHeight="1">
@@ -5416,7 +5432,7 @@
         <x:v>native-plugin/scripts/make-release.sh dry run before version bump</x:v>
       </x:c>
       <x:c r="I62" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="64" customHeight="1">
@@ -5445,7 +5461,7 @@
         <x:v>packaged 1-Install-PPTBridge-SK.command isolated HOME test</x:v>
       </x:c>
       <x:c r="I63" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="64" customHeight="1">
@@ -5474,7 +5490,7 @@
         <x:v>qa/obs-websocket-smoke.mjs plus hands-on OBS field test on 2026-07-16</x:v>
       </x:c>
       <x:c r="I64" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="64" customHeight="1">
@@ -5503,7 +5519,7 @@
         <x:v>qa/obs-feedback-runtime-smoke.mjs on 2026-07-16</x:v>
       </x:c>
       <x:c r="I65" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="64" customHeight="1">
@@ -5532,7 +5548,7 @@
         <x:v>qa/obs-websocket-smoke.mjs on 2026-07-18</x:v>
       </x:c>
       <x:c r="I66" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="64" customHeight="1">
@@ -5561,7 +5577,7 @@
         <x:v>native-plugin/scripts/make-release.sh; /tmp/pptbridge-v058-exact-final</x:v>
       </x:c>
       <x:c r="I67" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="64" customHeight="1">
@@ -5590,7 +5606,326 @@
         <x:v>OBS runtime-14 cleanup and SHA-256 verification on 2026-07-18</x:v>
       </x:c>
       <x:c r="I68" s="20" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-08-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="64" customHeight="1">
+      <x:c r="A69" s="20" t="str">
+        <x:v>T-065</x:v>
+      </x:c>
+      <x:c r="B69" s="20" t="str">
+        <x:v>INSTALL-001/PACK-001</x:v>
+      </x:c>
+      <x:c r="C69" s="20" t="str">
+        <x:v>macOS deployment target audit</x:v>
+      </x:c>
+      <x:c r="D69" s="20" t="str">
+        <x:v>Inspect the release Mach-O load commands and bundle plist after a clean Apple Silicon build.</x:v>
+      </x:c>
+      <x:c r="E69" s="20" t="str">
+        <x:v>The actual binary and Info.plist both support the documented macOS 12 minimum.</x:v>
+      </x:c>
+      <x:c r="F69" s="20" t="str">
+        <x:v>Found and fixed a release blocker: the previous binary encoded macOS 26.0. The v0.5.11 binary now encodes minos 12.0, SDK 26.5, arm64, and Info.plist minimum 12.0.</x:v>
+      </x:c>
+      <x:c r="G69" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H69" s="20" t="str">
+        <x:v>vtool -show-build, file, and PlistBuddy on 2026-08-25</x:v>
+      </x:c>
+      <x:c r="I69" s="20" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="64" customHeight="1">
+      <x:c r="A70" s="20" t="str">
+        <x:v>T-066</x:v>
+      </x:c>
+      <x:c r="B70" s="20" t="str">
+        <x:v>QA-001/LOAD-004/ROUTE-003/OSC-002/OSCFB-001</x:v>
+      </x:c>
+      <x:c r="C70" s="20" t="str">
+        <x:v>v0.5.11 standalone regression</x:v>
+      </x:c>
+      <x:c r="D70" s="20" t="str">
+        <x:v>Recompile release-object smoke binaries and run invalid input, registry, all OSC commands, all OSC feedback fields, PPTX/PDF render, presenter, navigation, cues, and embedded media.</x:v>
+      </x:c>
+      <x:c r="E70" s="20" t="str">
+        <x:v>All core behaviors pass against the final source with no crash or stale state.</x:v>
+      </x:c>
+      <x:c r="F70" s="20" t="str">
+        <x:v>Invalid input and registry passed; 8/8 OSC commands and 16/16 feedback fields passed; real 17-slide PPTX, 20-page PDF, and two-media fixture rendered and navigated correctly.</x:v>
+      </x:c>
+      <x:c r="G70" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H70" s="20" t="str">
+        <x:v>/tmp/pptbridge-macos-tests-v0511 on 2026-08-25</x:v>
+      </x:c>
+      <x:c r="I70" s="20" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="64" customHeight="1">
+      <x:c r="A71" s="20" t="str">
+        <x:v>T-067</x:v>
+      </x:c>
+      <x:c r="B71" s="20" t="str">
+        <x:v>QA-001</x:v>
+      </x:c>
+      <x:c r="C71" s="20" t="str">
+        <x:v>Sanitizer regression</x:v>
+      </x:c>
+      <x:c r="D71" s="20" t="str">
+        <x:v>Run invalid input, registry, OSC command/feedback, and real-deck render tests under ASan and UBSan.</x:v>
+      </x:c>
+      <x:c r="E71" s="20" t="str">
+        <x:v>No memory-safety or undefined-behavior diagnostic is emitted.</x:v>
+      </x:c>
+      <x:c r="F71" s="20" t="str">
+        <x:v>All selected sanitizer runs passed; macOS leak detection remains unsupported and was disabled explicitly.</x:v>
+      </x:c>
+      <x:c r="G71" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H71" s="20" t="str">
+        <x:v>ASAN_OPTIONS=detect_leaks=0:halt_on_error=1; UBSAN_OPTIONS=halt_on_error=1 on 2026-08-25</x:v>
+      </x:c>
+      <x:c r="I71" s="20" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="64" customHeight="1">
+      <x:c r="A72" s="20" t="str">
+        <x:v>T-068</x:v>
+      </x:c>
+      <x:c r="B72" s="20" t="str">
+        <x:v>SRC-001/SRC-002/ROUTE-001/PRES-001/LIVE-001/LIVE-003/LIVE-007</x:v>
+      </x:c>
+      <x:c r="C72" s="20" t="str">
+        <x:v>Full real OBS runtime, repeated</x:v>
+      </x:c>
+      <x:c r="D72" s="20" t="str">
+        <x:v>Run the complete visual WebSocket workflow twice in OBS 32.1.1 with two Program-routed decks, Presenter customization, cues, OSC feedback, resize modes, manual/auto live, reattach, final guard, black, and stop.</x:v>
+      </x:c>
+      <x:c r="E72" s="20" t="str">
+        <x:v>Every state is nonblank, correctly routed, reversible, and stable on repeat.</x:v>
+      </x:c>
+      <x:c r="F72" s="20" t="str">
+        <x:v>Two complete runs passed. Screenshots and pixel comparisons confirmed source routing, Presenter layout, 16 OSC status fields, live lifecycle, final-slide guard, and black restore.</x:v>
+      </x:c>
+      <x:c r="G72" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H72" s="20" t="str">
+        <x:v>qa/obs-websocket-smoke.mjs; /tmp/pptbridge-obs-runtime-20260825-pass2</x:v>
+      </x:c>
+      <x:c r="I72" s="20" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="64" customHeight="1">
+      <x:c r="A73" s="20" t="str">
+        <x:v>T-069</x:v>
+      </x:c>
+      <x:c r="B73" s="20" t="str">
+        <x:v>HOTKEY-004/CLICKER-001/CLICKER-002/CLICKER-003</x:v>
+      </x:c>
+      <x:c r="C73" s="20" t="str">
+        <x:v>Real macOS clicker and typing isolation</x:v>
+      </x:c>
+      <x:c r="D73" s="20" t="str">
+        <x:v>Focus a key-receiver app, send Left, Right, Space, PageDown, and PageUp while clicker capture is enabled, and inspect the Program deck.</x:v>
+      </x:c>
+      <x:c r="E73" s="20" t="str">
+        <x:v>Normal editing keys reach the focused app; PageDown/PageUp control only PPTBridge and are suppressed from that app.</x:v>
+      </x:c>
+      <x:c r="F73" s="20" t="str">
+        <x:v>Left/Right/Space reached the focused app and did not move the deck. PageDown moved the Program deck, PageUp restored it, and neither reached the focused app.</x:v>
+      </x:c>
+      <x:c r="G73" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H73" s="20" t="str">
+        <x:v>qa/obs-macos-clicker-runtime-smoke.mjs on 2026-08-25</x:v>
+      </x:c>
+      <x:c r="I73" s="20" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="64" customHeight="1">
+      <x:c r="A74" s="20" t="str">
+        <x:v>T-070</x:v>
+      </x:c>
+      <x:c r="B74" s="20" t="str">
+        <x:v>MEDIA-001/AUDIO-001/AUDIO-003</x:v>
+      </x:c>
+      <x:c r="C74" s="20" t="str">
+        <x:v>Installed embedded-media audio</x:v>
+      </x:c>
+      <x:c r="D74" s="20" t="str">
+        <x:v>Run a synthetic 880 Hz embedded-media fixture through installed OBS with enabled, disabled, unity, and -20 dB settings.</x:v>
+      </x:c>
+      <x:c r="E74" s="20" t="str">
+        <x:v>Audio appears once at the parent source, disabling is silent, and gain is exact.</x:v>
+      </x:c>
+      <x:c r="F74" s="20" t="str">
+        <x:v>Enabled recording contained the tone, disabled output was silent, and -20 dB produced the exact 0.1 amplitude multiplier without duplicate gain.</x:v>
+      </x:c>
+      <x:c r="G74" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H74" s="20" t="str">
+        <x:v>qa/obs-audio-runtime-smoke.mjs and recording analysis on 2026-08-25</x:v>
+      </x:c>
+      <x:c r="I74" s="20" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="64" customHeight="1">
+      <x:c r="A75" s="20" t="str">
+        <x:v>T-071</x:v>
+      </x:c>
+      <x:c r="B75" s="20" t="str">
+        <x:v>INSTALL-004/PACK-001</x:v>
+      </x:c>
+      <x:c r="C75" s="20" t="str">
+        <x:v>Deterministic v0.5.11 Apple Silicon package</x:v>
+      </x:c>
+      <x:c r="D75" s="20" t="str">
+        <x:v>Build the final ZIP twice, verify both SHA-256 values, inspect all members, architecture, minimum macOS, version, signatures, duplicates, and junk.</x:v>
+      </x:c>
+      <x:c r="E75" s="20" t="str">
+        <x:v>Both package runs are byte-identical and contain only the documented installer and support files.</x:v>
+      </x:c>
+      <x:c r="F75" s="20" t="str">
+        <x:v>Both runs produced SHA-256 3f6b3bf7c646eef2a88c548e4d27c0af3aeac8c34e3fb63fd514e652ad67dea2. ZIP has 20 entries, no duplicate/junk paths, arm64 0.5.11 plugin, minos 12.0, and valid ad-hoc signature.</x:v>
+      </x:c>
+      <x:c r="G75" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H75" s="20" t="str">
+        <x:v>native-plugin/scripts/make-release.sh on 2026-08-25</x:v>
+      </x:c>
+      <x:c r="I75" s="20" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="64" customHeight="1">
+      <x:c r="A76" s="20" t="str">
+        <x:v>T-072</x:v>
+      </x:c>
+      <x:c r="B76" s="20" t="str">
+        <x:v>INSTALL-001/INSTALL-004</x:v>
+      </x:c>
+      <x:c r="C76" s="20" t="str">
+        <x:v>Exact ZIP installation and safety</x:v>
+      </x:c>
+      <x:c r="D76" s="20" t="str">
+        <x:v>Install the exact final ZIP into an isolated HOME and the real user plugin path, compare executable bytes, then rerun the installer while OBS is open.</x:v>
+      </x:c>
+      <x:c r="E76" s="20" t="str">
+        <x:v>Installer copies an identical valid bundle when OBS is closed and refuses replacement without changing bytes when OBS is running.</x:v>
+      </x:c>
+      <x:c r="F76" s="20" t="str">
+        <x:v>Isolated and real installs succeeded; installed bundle is 0.5.11 arm64 minos 12.0 and byte-identical. OBS-open run exited 1 and preserved SHA-256 90ba47b38dfd758e945b7e70c1f33c1ed2e4ef75367bb9d626ca032400992f9b.</x:v>
+      </x:c>
+      <x:c r="G76" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H76" s="20" t="str">
+        <x:v>Final packaged 1-Install-PPTBridge-SK.command on 2026-08-25</x:v>
+      </x:c>
+      <x:c r="I76" s="20" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="64" customHeight="1">
+      <x:c r="A77" s="20" t="str">
+        <x:v>T-073</x:v>
+      </x:c>
+      <x:c r="B77" s="20" t="str">
+        <x:v>SRC-001/SRC-002/NAV-001</x:v>
+      </x:c>
+      <x:c r="C77" s="20" t="str">
+        <x:v>Exact installed plugin smoke</x:v>
+      </x:c>
+      <x:c r="D77" s="20" t="str">
+        <x:v>Launch OBS from the packaged installer, create temporary Slide and Presenter inputs, capture both, press Next and Previous, and clean all QA objects.</x:v>
+      </x:c>
+      <x:c r="E77" s="20" t="str">
+        <x:v>Both source kinds render nonblank frames; navigation changes and restores output; cleanup leaves user scenes intact.</x:v>
+      </x:c>
+      <x:c r="F77" s="20" t="str">
+        <x:v>Installed 0.5.11 produced 399814-byte Slide and 214248-byte Presenter screenshots; Next changed the frame and Previous restored the original hash. Temporary inputs/scenes were removed.</x:v>
+      </x:c>
+      <x:c r="G77" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H77" s="20" t="str">
+        <x:v>OBS WebSocket exact-install smoke on 2026-08-25</x:v>
+      </x:c>
+      <x:c r="I77" s="20" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="64" customHeight="1">
+      <x:c r="A78" s="20" t="str">
+        <x:v>T-074</x:v>
+      </x:c>
+      <x:c r="B78" s="20" t="str">
+        <x:v>LIVE-001/LIVE-003/LIVE-007/NAV-003</x:v>
+      </x:c>
+      <x:c r="C78" s="20" t="str">
+        <x:v>Final v0.5.11 PowerPoint Live lifecycle</x:v>
+      </x:c>
+      <x:c r="D78" s="20" t="str">
+        <x:v>Run the release-object live smoke on a real 17-slide PPTX after the deployment-target rebuild.</x:v>
+      </x:c>
+      <x:c r="E78" s="20" t="str">
+        <x:v>Start, first/next/last, repeated Next at final, Previous, black toggle/restore, and Stop all succeed.</x:v>
+      </x:c>
+      <x:c r="F78" s="20" t="str">
+        <x:v>Live mode started in 4166 ms; all navigation/final-guard/black checks passed and Stop closed the slideshow cleanly.</x:v>
+      </x:c>
+      <x:c r="G78" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H78" s="20" t="str">
+        <x:v>/tmp/pptbridge-macos-tests-v0511/live_start_smoke on 2026-08-25</x:v>
+      </x:c>
+      <x:c r="I78" s="20" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="64" customHeight="1">
+      <x:c r="A79" s="20" t="str">
+        <x:v>T-075</x:v>
+      </x:c>
+      <x:c r="B79" s="20" t="str">
+        <x:v>QA-001</x:v>
+      </x:c>
+      <x:c r="C79" s="20" t="str">
+        <x:v>NDI/DistroAV coexistence</x:v>
+      </x:c>
+      <x:c r="D79" s="20" t="str">
+        <x:v>Start installed OBS 32.1.1 with PPTBridge 0.5.11 and inspect module/runtime logs.</x:v>
+      </x:c>
+      <x:c r="E79" s="20" t="str">
+        <x:v>PPTBridge and DistroAV load together without disabling NDI output.</x:v>
+      </x:c>
+      <x:c r="F79" s="20" t="str">
+        <x:v>PPTBridge registered successfully; DistroAV 6.2.1 initialized NDI SDK 6.3.2.0 and started both Main and Preview outputs.</x:v>
+      </x:c>
+      <x:c r="G79" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H79" s="20" t="str">
+        <x:v>OBS log 2026-08-25 14-04-36.txt</x:v>
+      </x:c>
+      <x:c r="I79" s="20" t="str">
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5599,13 +5934,13 @@
     <x:mergeCell ref="A2:N2"/>
   </x:mergeCells>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="G5:G68">
+    <x:dataValidation type="list" sqref="G5:G79">
       <x:formula1>"Pass,Fail,Not Run,Blocked,Retest Required"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re303c10296e44faa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2385bdc8e5c4de8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5860,22 +6195,54 @@
         <x:v>Retested Pass</x:v>
       </x:c>
     </x:row>
+    <x:row r="11" ht="72" customHeight="1">
+      <x:c r="A11" s="20" t="str">
+        <x:v>ISS-007</x:v>
+      </x:c>
+      <x:c r="B11" s="20" t="str">
+        <x:v>INSTALL-001/PACK-001</x:v>
+      </x:c>
+      <x:c r="C11" s="20" t="str">
+        <x:v>Closed</x:v>
+      </x:c>
+      <x:c r="D11" s="20" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E11" s="20" t="str">
+        <x:v>macOS Compatibility</x:v>
+      </x:c>
+      <x:c r="F11" s="20" t="str">
+        <x:v>The release binary encoded a macOS 26.0 deployment target even though the bundle and documentation advertised macOS 12.</x:v>
+      </x:c>
+      <x:c r="G11" s="20" t="str">
+        <x:v>vtool -show-build on installed v0.5.10 and first v0.5.11 candidate</x:v>
+      </x:c>
+      <x:c r="H11" s="20" t="str">
+        <x:v>Keep the Mach-O minos assertion in every Apple Silicon release check.</x:v>
+      </x:c>
+      <x:c r="I11" s="20" t="str">
+        <x:v>CMake now sets CMAKE_OSX_DEPLOYMENT_TARGET=12.0 before project() when no explicit target is supplied. The rebuilt 0.5.11 binary and packaged installer both report minos 12.0.</x:v>
+      </x:c>
+      <x:c r="J11" s="20" t="str">
+        <x:v>Retested Pass</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:N1"/>
     <x:mergeCell ref="A2:N2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="C5:C10">
+    <x:dataValidation type="list" sqref="C5:C11">
       <x:formula1>"Open,Fixed,Retesting,Closed,Deferred"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D5:D10">
+    <x:dataValidation type="list" sqref="D5:D11">
       <x:formula1>"P0,P1,P2,P3"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R886a0d676c344ef1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7bf93106c4a458d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>